<commit_message>
stricter constraints on AAV/LV, added URLs to source
</commit_message>
<xml_diff>
--- a/onlygemini_results.xlsx
+++ b/onlygemini_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,7 +538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "webSearchQueries": ["WuXi Advanced Therapies annual reports", "WuXi Advanced Therapies investor presentations", "WuXi Advanced Therapies earnings releases", "WuXi Advanced Therapies regulatory filings", "WuXi Advanced Therapies manufacturing sites", "WuXi Advanced Therapies advanced therapy revenue", "WuXi Advanced Therapies CDMO revenue", "WuXi AppTec annual report advanced therapies", "WuXi Advanced Therapies AAV LV manufacturing", "WuXi Advanced Therapies gene therapy manufacturing", "WuXi Advanced Therapies stem cell manufacturing"]}</t>
+          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "groundingChunks": [{"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFl_vECPci4yVIil4DtYinFlS5juzqTA8WNKIIuctyiqvuczIhlid52PEdFukGzN2JkQGqxspkiwfJCqynjPcg6OG_jFzM67Hn9zk2ebRl3HYqcPleYgZ_VDua1LsPrBpeyjqOd", "title": "firstwordpharma.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGTru9O__3JKDuerPXcLgDihHy08H0iVJE--ePGyKCbjVvNIPwnOAHe-gkztlc3ox_uBXedWVrmokpzQI-VOorBhuB0F7z7Bb9IeDanz4nEnzJZjCyN6KV4dv2u6ToOifJeAXSQj2s6eioXEQFHlJOXsDoH1GMVU4Mf", "title": "pharmasource.global"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEizzEcXgFlSKvxGOJ_hy7JOObi5_jHH02z6BdFVI5nfudbNi43ZCWuNXxhpI1QseNVri-Qz_dAP2ZwQEfOIcIJfj9zZBFNhr-ahvszQA4NBRljlSN0Zi5C0jn7x1uSKYH8zJxB0QlGsA8=", "title": "wuxiapptec.com"}}], "groundingSupports": [{"segment": {"startIndex": 15530, "endIndex": 15588, "text": "This figure is used as the total advanced therapy revenue."}, "groundingChunkIndices": [0]}, {"segment": {"startIndex": 15588, "endIndex": 15819, "text": "\",\n\"This total revenue is entirely attributable to advanced therapy manufacturing modalities, as WuXi Advanced Therapies is a Contract Testing, Development, and Manufacturing Organization (CTDMO) focused on cell and gene therapies."}, "groundingChunkIndices": [1, 2]}], "webSearchQueries": ["WuXi Advanced Therapies annual report", "WuXi Advanced Therapies investor presentation", "WuXi Advanced Therapies earnings release", "WuXi Advanced Therapies regulatory filings", "WuXi Advanced Therapies manufacturing sites", "WuXi Advanced Therapies AAV manufacturing", "WuXi Advanced Therapies lentiviral vector manufacturing", "WuXi Advanced Therapies gene therapy manufacturing revenue", "WuXi Advanced Therapies cell therapy manufacturing revenue", "WuXi Advanced Therapies CDMO revenue", "WuXi Advanced Therapies advanced therapies revenue", "WuXi Advanced Therapies 2023 revenue", "WuXi Advanced Therapies 2024 revenue", "WuXi Advanced Therapies 2025 revenue", "WuXi AppTec advanced therapies business unit revenue", "WuXi AppTec annual report advanced therapies", "WuXi Advanced Therapies capabilities AAV LV", "WuXi Advanced Therapies capabilities stem cell"]}</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>["The revenue figures for 'WuXi Advanced Therapies' are based on the reported performance of the WuXi AppTec Advanced Therapies unit (primarily its US and UK operations) before its divestment to Altaris, LLC in late 2024/early 2025. This unit represented the core of WuXi Advanced Therapies' manufacturing business.", "An exchange rate of 1 USD = 7.2 RMB was used for currency conversions.", "The total advanced therapy manufacturing revenue for 2024 (RMB 1.32 billion / $183.33 million USD) was used as the base for attribution, as it is the most recent comprehensive figure for the unit before divestment.", "AAV/LV Viral Vector Manufacturing revenue is estimated at 60% of the total advanced therapy revenue, given the strong and explicit evidence of AAV/LV technologies (TESSA, LentiVEX) and dedicated manufacturing platforms.", "Stem Cell Therapeutic Manufacturing revenue is estimated at 10% of the total advanced therapy revenue, inferred from the presence of a 'non-viral cell therapy plant' and the subsequent merger with Minaris Regenerative Medicine, acknowledging that explicit 'stem cell' revenue is not separately reported.", "The remaining 30% of the total advanced therapy revenue is attributed to other Gene Therapy Manufacturing (excluding AAV/LV and stem cell, but including other viral vectors and gene-modified cell therapies like CAR-T that are not specifically AAV/LV).", "The 'gene_therapy_revenue_estimate' in the summary includes both AAV/LV and other gene therapy manufacturing, as per the hierarchy rule that AAV/LV is a subset of Gene Therapy."]</t>
+          <t>["The most relevant revenue for 'WuXi Advanced Therapies' is the RMB 1.32 billion (approximately USD 182.57 million) reported for its US and UK operations in 2024, as these were the divested entities that constituted WuXi Advanced Therapies. This figure is used as the total advanced therapy revenue.", "This total revenue is entirely attributable to advanced therapy manufacturing modalities, as WuXi Advanced Therapies is a Contract Testing, Development, and Manufacturing Organization (CTDMO) focused on cell and gene therapies.", "The total advanced therapy revenue is apportioned between Gene Therapy Manufacturing and Stem Cell Therapeutic Manufacturing. Based on the extensive descriptions of both viral vector (gene therapy) and cell therapy capabilities, a split of 50-70% for Gene Therapy and 30-50% for Stem Cell Therapy is inferred. This split is used to derive the range_low, range_high, and value for these buckets.", "Within Gene Therapy Manufacturing, AAV/LV Viral Vector Manufacturing is estimated to account for 70-90% of the revenue, given the prominent mention of TESSA\u00ae and XLenti\u2122 technologies and dedicated platforms for AAV and LV. This sub-split is used to derive the range_low, range_high, and value for the AAV/LV bucket."]</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>[{"source": "WuXi AppTec 2023 Annual Report", "page": "Page 23", "keywords": ["WuXi ATU", "revenue", "RMB1.31 billion", "development, testing and manufacturing services", "64 projects", "cell and gene therapy"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 181.94, "range_low": null, "range_high": null}, "notes": "Reported revenue for WuXi ATU in 2023 was RMB 1.31 billion, which converts to approximately $181.94 million USD. This represents the overall advanced therapies business unit."}, {"source": "WXAT 2024 Annual Results Presentation", "page": "Page 23", "keywords": ["Discontinued Operations", "revenue of RMB1.32 billion in 2024", "advanced therapies"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 183.33, "range_low": null, "range_high": null}, "notes": "WuXi AppTec reported that its divested Advanced Therapies operations (US and UK) contributed RMB 1.32 billion in revenue in 2024, which converts to approximately $183.33 million USD. This is the most recent and comprehensive reported revenue for the advanced therapies manufacturing unit before its divestment."}, {"source": "BRIEF: WuXi AppTec sells advanced therapies units in U.K. and U.S.", "page": "", "keywords": ["Advanced Therapies and Oxford Genetics", "980 million yuan ($134 million) in revenue", "first 11 months of this year"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": 134.0, "range_low": null, "range_high": null}, "notes": "Reported revenue for Advanced Therapies and Oxford Genetics for the first 11 months of 2024 was approximately $134 million USD. This supports the overall scale of the advanced therapies business."}, {"source": "WuXi Advanced Therapies - PharmaSource", "page": "", "keywords": ["CTDMO", "cell and gene therapy innovation", "TESSA\u00ae AAV production", "XOFLX\u2122 cell lines", "Manufacturing: Clinical and commercial manufacturing for cell and gene therapies"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 110.0, "range_low": null, "range_high": null}, "notes": "Explicit mention of AAV production technology (TESSA) and viral vector manufacturing capabilities. This forms a significant portion of gene therapy revenue."}, {"source": "Regulatory Archives - Advanced Therapies", "page": "", "keywords": ["GMP lentivirus manufacturing", "CAR-T cell therapy product", "process development and manufacturing of LVV"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Direct evidence of lentiviral vector (LVV) manufacturing for CAR-T cell therapy, which falls under AAV/LV viral vector manufacturing."}, {"source": "WuXi Advanced Therapies Launches New World-Class AAV Vector Suspension Platform", "page": "", "keywords": ["AAV Vector Suspension Platform", "AAV vector production", "gene therapy development, manufacturing and release", "scalability that range up to 1000L"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Announcement of a dedicated AAV vector suspension platform, highlighting strong capabilities in AAV manufacturing."}, {"source": "The Future of AAV Gene Therapy Is Scalable - BioProcess International", "page": "", "keywords": ["Oxgene", "adenoassociated virus (AAV) and lentivirus platforms", "TESSA and LentiVEX platforms/technologies", "scale processes up to good manufacturing practice (GMP) manufacturing through to commercial supply"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Acquisition of Oxgene brought AAV and lentivirus platforms, confirming strong capabilities in viral vector manufacturing for gene therapies."}, {"source": "WuXi Advanced Therapies Enters Licensing Agreement with Janssen - Contract Pharma", "page": "", "keywords": ["TESSA technology", "produce 10 times more adeno-associated viral (AAV) vectors", "large scale AAV manufacturing"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Licensing of TESSA technology for AAV vector production demonstrates advanced capabilities and industry recognition in this specific modality."}, {"source": "WuXi Advanced Therapies - PharmaSource", "page": "", "keywords": ["CTDMO", "cell and gene therapy innovation", "comprehensive solutions for the discovery, development, and commercialisation of cell and gene therapies", "Manufacturing: Clinical and commercial manufacturing for cell and gene therapies"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 165.0, "range_low": null, "range_high": null}, "notes": "Broad statements about cell and gene therapy manufacturing services, encompassing various gene therapy modalities."}, {"source": "WuXi Advanced Therapies Locations - Contract Research Map", "page": "", "keywords": ["Contract Manufacturing &amp; Development and Laboratory Testing Services for Cell, Gene, Protein and Viral-Based Therapeutics", "cGMP manufacture of advanced gene and cell therapies (autologous &amp; allogeneic)"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Confirms cGMP manufacturing for both gene and cell therapies, including autologous and allogeneic approaches, which are common in gene therapy."}, {"source": "Regulatory Archives - Advanced Therapies", "page": "", "keywords": ["integrated platforms to transform the discovery, development, testing, manufacturing, and commercialization of cell and gene therapies"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights the end-to-end service offering for cell and gene therapies."}, {"source": "WuXi AppTec selling CGT unit as BIOSECURE continues to play out", "page": "", "keywords": ["late phase/commercial viral manufacturing facility", "non-viral cell therapy plant", "process development/early phase clinical manufacturing site"], "bucket": "stem_cell", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 18.33, "range_low": null, "range_high": null}, "notes": "The mention of a 'non-viral cell therapy plant' suggests capabilities beyond gene-modified cells, which could include stem cell manufacturing. This is further supported by the subsequent combination with Minaris Regenerative Medicine."}, {"source": "WuXi Advanced Therapies, Minaris Regenerative Medicine combine to form new CDMO", "page": "", "keywords": ["Minaris Regenerative Medicine", "U.S. and U.K. operations of WuXi AppTec's Advanced Therapies Unit", "global cell therapy CDMO and testing partner"], "bucket": "stem_cell", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "The merger with Minaris Regenerative Medicine, a company focused on regenerative medicine (often involving stem cells), indicates that the cell therapy capabilities of WuXi Advanced Therapies likely included stem cell manufacturing."}]</t>
+          <t>[{"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG0h3ymjlaMKFjVahY8YMjAIaxhEEdy1-EnWbWvQhONS0EJOzL3PYRHBgTyadw3E5HJE6f9liL8WfQY6XH03awR6COskLwzrMnPHrB1tT7vnyFK2yVlDkydt5lGxZNBl6eDC_1KlofJ8J5LuB8dHKAHUr15rH66gqZNuXrP8wCu8rOkpPnFzULqg-XwPUf03HM=", "source": "BRIEF: WuXi AppTec sells advanced therapies units in U.K. and U.S. - Bamboo Works", "page": "", "keywords": ["Advanced Therapies", "Oxford Genetics", "revenue", "980 million yuan", "134 million"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 134.0, "range_low": null, "range_high": null}, "notes": "Revenue for WuXi Advanced Therapies and Oxford Genetics for the first 11 months of 2024, approximately $134 million."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFl_vECPci4yVIil4DtYinFlS5juzqTA8WNKIIuctyiqvuczIhlid52PEdFukGzN2JkQGqxspkiwfJCqynjPcg6OG_jFzM67Hn9zk2ebRl3HYqcPleYgZ_VDua1LsPrBpeyjqOd", "source": "WuXi AppTec Revenue and Profit Achieved Steady QoQ Growth in 2024, Meeting Full-year Guidance", "page": "", "keywords": ["WuXi ATU", "US and UK based operations", "Discontinued Operations", "revenue", "RMB1.32 billion", "2024"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 182.57, "range_low": null, "range_high": null}, "notes": "The US and UK based operations of WuXi Advanced Therapies (WuXi ATU), classified as Discontinued Operations, collectively contributed RMB1.32 billion in revenue in 2024. Converted to USD using an approximate 2024 exchange rate of 7.23 RMB/USD, this is $182.57 million."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGTru9O__3JKDuerPXcLgDihHy08H0iVJE--ePGyKCbjVvNIPwnOAHe-gkztlc3ox_uBXedWVrmokpzQI-VOorBhuB0F7z7Bb9IeDanz4nEnzJZjCyN6KV4dv2u6ToOifJeAXSQj2s6eioXEQFHlJOXsDoH1GMVU4Mf", "source": "WuXi Advanced Therapies - PharmaSource", "page": "", "keywords": ["CTDMO", "cell and gene therapy", "manufacturing", "TESSA\u00ae AAV production", "XOFLX\u2122 cell lines"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies is a global CTDMO supporting cell and gene therapy innovation, with capabilities in manufacturing for cell and gene therapies, including TESSA\u00ae AAV production and XOFLX\u2122 cell lines."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGWPrJEG7dIjEmccWL-Qsc1ruIQ07S2BnJzR93nIkW3hZ-vWHZfSZJK-Ti9e0NZJ0Kfr_xS2I-qWsO6v6IuZN-ij6VpNs8DZ8nMqaEEnXDRXSSAF8VBXNPp0vMzAMu3a_sOdW_ZIEURIaLzCzbY", "source": "WuXi Advanced Therapies: Revenue, Competitors, Alternatives - Growjo", "page": "", "keywords": ["CDMO", "cell, gene, protein and viral-based therapies"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies is a CDMO pioneering the expedited development and commercialization of cell, gene, protein and viral-based therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHppGfSfD189g__FvBuJdw6RSsLTZ7JeNWaa_j09wda0w4Ozzeru7LHTCR-2GaxzhP2rCLApIFvORX_NvlEO-DoYAba2QDa3gvO7ZZOCYXOIbr_rmllTMMJ3n9TsLuPCnSW", "source": "AAV Archives - Advanced Therapies", "page": "", "keywords": ["TESSA\u00ae technology", "AAV manufacturing", "GMP grade", "AAV vectors"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies developed TESSA\u00ae technology for transfection-free, scalable, GMP-grade AAV vector production."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF4gCl72wtU3y5JL8GqK04pmequ-2dXwQ28TJyqjQVS4lRwPd6sip4AQhizxdHhMOBnG2pjfvxnq6nt638Si884B-qjPCmwGynFbEkRhP7iu-DkUOZy559XwijB77EF8H9us7iY8sYMuK1krytZxP8pvby-eLRdLnvf8wz7kfw8bblKTIpn8wFk9eWlCgwUbKo1TEAptfr47UoiBOI0b-z4H312DJjQM7KwUKihFdAl_0MH7g4AX2-ZIUc0K_IsYODX4mw=", "source": "WuXi Advanced Therapies Launches New World-Class AAV Vector Suspension Platform", "page": "", "keywords": ["AAV Vector Suspension Platform", "AAV vector production", "cell and gene therapy development", "manufacturing"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies launched an integrated AAV Vector Suspension Platform for cell and gene therapy development, manufacturing, and release."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGEQq5-eloujgF9KXyZHFmrhAd8rLn2lEBYUaWj_Ecnqk-TqCgrYHB3M1YBgQisetGDiyfMncHE8NeaLwH38Q5PlUqBL-22ZdWS_50KmSmAabKPxzQlWz94lNHYvf9XqL1biv69Gfh1Kszn7MIY0_RYOjfWZvtD57IyLuvGO0xnrAOGd7CwOIIJu0dZHXmgTe9okUPOLsbmRty39NJA1oyH_FNLj0TU1Xc=", "source": "Developing a Platform for Large-Scale Lentiviral Manufacture - BioProcess International", "page": "", "keywords": ["lentiviral vectors", "gene delivery tools", "cell and gene therapies", "lentiviral suspension manufacturing platform"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies developed a lentiviral suspension manufacturing platform for large-scale lentiviral vector manufacture for cell and gene therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFV9-lfUfOiLthf4gBi1r8ST3zsRUGcD4NusWNnAGbid8I43CLg1pRQNqB6A3tR40ouUWAeR_8A7y-TgfXJHm1lE9HXjfFMin_fgv-J6qKgA55TmOyoDVXU9KRol6uHo5EhvDYbURDB7BTQSkBWjWmn1O5yAUOMzrqSTmCNm-5D4g==", "source": "WuXi Advanced Therapies Locations - Contract Research Map", "page": "", "keywords": ["cGMP manufacturing", "cell, gene, protein and viral-based therapeutics", "autologous &amp; allogeneic"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies provides cGMP manufacturing for cell, gene, protein and viral-based therapeutics, including autologous &amp; allogeneic cell and gene therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGY1stdygtL_ag9tq69b_o6_e7QHSI-DNXvEUoMytfio_gOjcWlSP4D-ZJCEtBeGo5egCW09qey8SeAwfoAQtBuSirWpSNVCV-JNsmrqZUZS7PrKiuxYKaLtglJex04qqpFqDv_PX7k7x_ntDj7azFZAKDPtgOppR-RHR32aLuikzBmR7pqkUtCDF2i31eM627GiqwX0Ae27ggWXIM6Ilb6vqqj6HlBqyglm9X4yJkL5aiWrmIWTaALLIGPgd0=", "source": "With BIOSECURE Act looming, WuXi AppTec sustains another revenue decline while still attracting new business - Fierce Biotech", "page": "", "keywords": ["WuXi Advanced Therapies", "cell and gene therapies", "manufacture"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies offers services to help partners advance and manufacture their cell and gene therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFhJYDu3UwWxiV9bQIsOGXZN6mqoCKXOxL-_X6N8g_xJhcaOUFAR0_OeG8IPj4MeOOXc8Fih9fR1h0ymObnlD3EmRUyIZRuc2G3ntpvRskVZ-IbDhOcnEEWeyWuCmC_N0ijbsO28dQLfzM33F9fpJo0jS58c957AAC1laAXxf_OGOeVigMaFQSfT5VWaF9dD0ppP-WmtQ7d7Zs6NNAIqeMSJIY7omrWp7xicTkAkDsj0KX9rawAnk=", "source": "Manufacture of lentiviral vectors using suspension Packaging and Producer cell lines yields titres comparable to transient process - Minaris Advanced Therapies", "page": "1", "keywords": ["Lentiviral vectors", "LVV", "cell and gene therapy", "vector manufacturing", "LVV Packaging and Producer cell lines"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies (OXGENE) developed LVV Packaging and Producer cell lines to reduce vector manufacturing cost and process variability for lentiviral vectors in cell and gene therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGuY-wrZZrFzkwk6qQFlae-91aqYHCOHevzjwCEolBsG0yuDQAdFy7hB9ptFyW403nw9y-qb4r9S_TpZ91x8aroOYxvnyqE9MYborRXeO3X5GUSlXCnLf38lT-z8t5wBWVSVz90rPcRowhxP4J0NubqX_vqUWquJE5XzeCey0C3Smn4R_RY4uDTZWFEVSQs6Ricl2tFDOI=", "source": "The Future of AAV Gene Therapy Is Scalable - BioProcess International", "page": "", "keywords": ["AAV", "lentivirus platforms", "TESSA", "LentiVEX", "GMP manufacturing"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies, through the acquisition of Oxgene, utilizes TESSA and LentiVEX platforms for AAV and lentivirus GMP manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFQWjsEhhAr_SWXth3mJRB6QMbolu0HEhTuubAm-h15TplNGc5rzBh6KbaXM2EV29xy-72GQ83nFpWJRIm83aS3E2z37Uhf3Mqy5N5ahh154z97xphIUsDdVJQuJsbGDaIUJ9WqKj66nhM=", "source": "WuXi ATU Announces Licensing Agreement with Janssen for TESSA\u2122 Technology", "page": "", "keywords": ["TESSA\u2122 technology", "AAV vectors", "AAV manufacturing", "gene therapies"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi ATU licensed its TESSA\u2122 technology for AAV vector manufacturing to Janssen, highlighting its high-performance system for gene therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEw6JP2weDzmzab_LG0mYrTkrrHKsYMCz-j7xmeQX0xShhwWq2rOvDT3PH4wnN8ViZUCXSRPDIj3bGzEuwb7aJTtIrOUpWB4vQTrp4UIVYjQqqRQFEEegth0EI08t2pYsgC5LZc4M2ByxyMrCJBWydJPH5A0JhiOjuNBdTWBHR4WbBXXYTK-L_4cGRIUO-aIA0iG3lL5ASznZsOCN7VLhJZNAtWt1YcEo1yU_L3ANt_ugdX2llXwUWKG2IW2Jxsgank7zmYi-c4DPL-qVIyOx4U75UKVhyW2-w=", "source": "WuXi ATU Opens New Manufacturing Facility to Further Enhance Its CTDMO Services for Global Customers - PR Newswire", "page": "", "keywords": ["viral vectors", "cell therapies", "manufacturing", "Lin-gang, Shanghai"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi ATU opened a new facility in Lin-gang, Shanghai, offering integrated development, manufacturing, and testing services for viral vectors and cell therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEqVmpsLL1K_eV_W4G7g6hPNPm_kkTpG7nW6r-YNjTiQ5jw-_o5Oda_izbsAJB5VJaydfuw-csOi6KnLsULammzeVpjnU7NN4djvFsFLNu8yCr52edD36PA_RtBccaBXk3ZoKSnbxc=", "source": "WuXi Advanced Therapies - YouTube", "page": "", "keywords": ["viral vector manufacturing", "cell therapy manufacturing", "AAV", "Lenti"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies performs viral vector manufacturing (AAV and Lenti) and cell therapy manufacturing across its sites."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHlV00RXafRPm5hPcfvIpethm7mbQJat6lFD2xayv7fKiqzU-srgFVCbtfuMBgS627UUtBgUIHJBD1xrD64rrld8b4bj_YXC67XZvQGSi8oaPOZ6CQxoEHe94l2JIpm_63i-4qMuwNWotjFXlmcVPrd4HqfZXOWxfccXjvS9CfzBNl9tlTu9xzBtpUFy7XIXiceE4P5ShOjcl1BADErac-a0gDHIgd4SX1IfEhaPm6Q8RAJVYalYVrmxXRXHqs8rIPPxjPJM0H8E1ZUR3CDpOV8H1Lk6zfB27o=", "source": "Interius BioTherapeutics Announces Successful Manufacturing Partnership with WuXi Advanced Therapies - PR Newswire", "page": "", "keywords": ["lentiviral vector manufacturing", "GMP manufacturing", "CAR T cells"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies partnered with Interius BioTherapeutics for GMP manufacturing of lentiviral vectors for CAR T cell therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEd-fPBaKRbvht8yX3yu3M0L4nxRT1YZsZjxAISqID6eKEHJMH9r-Ilwbpty28swmsh59qaFJqi8kQqB5YImm0mzMlgB8OyRXgBkoHOoIkjxAMSgq3go_2nPWwZRB4xoglT4jjyHhcTKBa2PJdxzuRU1e-805Azw2BDMrul6tQ1PFNPaWItONv57VH9eEt3d1TtWal3rXeVKxn67fifcYHOvZV37VpbHVQ=", "source": "2022-09 WuXi ATU Lenti Plasmids - Minaris Advanced Therapies", "page": "2", "keywords": ["cell and gene therapy manufacturing solutions", "viral vector production", "Lentiviral plasmids", "GMP grade"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies offers proprietary cell and gene therapy manufacturing solutions for high-titre, scalable, and cost-effective viral vector production, including GMP-grade lentiviral plasmids."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHFEYC_I2-yt5Rd6dCgKd2lKddaeib8JrTeVAPJM2x8JPkvR3nc-jIvAncBK_Vxjq_gRck06Jk3Ll5SNcUfNztTSJPz45kYWeRswRXhUWtUHojZ3Ow1zJvE7Scr4e6I2I8IF_FdBkaMGWhR2ASeDn_vKMbCGSAmhJiDmWCofkZpLVo2YKJAGHobigFR7DfXLSKMZ4ohzoU19wogLCAI6W655tKvPSuxAAV0CXHYVJ_rMo2Ef6pRQLhy9xqaD4O2CaqmhVQbWqTXMyhuyPUyWiCui1jxH-vLrIo=", "source": "WuXi Advanced Therapies' Philadelphia Site Approved by FDA to Start Manufacturing Iovance's Melanoma T-cell Therapy", "page": "", "keywords": ["Philadelphia Site", "FDA Approved", "Manufacturing", "T-cell Therapy"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies' Philadelphia site received FDA approval for manufacturing Iovance's melanoma T-cell therapy, indicating capabilities in cell therapy manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFGG1nbHsNaG8_T4NlJMGjf_hTjzOqRFwPFJNrzC0f_E-JWSqeYRBJ8U-He3M1oNjfqxWnwTc9pxPjCnob4uXgl0vdg9Z0NlkLxCGzv641rhBrI_PPfpMF-iocQenylfPfsE1YM3oVOpg==", "source": "Regulatory Archives - Advanced Therapies", "page": "", "keywords": ["CTDMO", "cell and gene therapies", "TESSA technology for AAV manufacturing", "XLenti stable solutions for lentiviral manufacturing"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi Advanced Therapies is a CTDMO offering integrated platforms for cell and gene therapies, including TESSA technology for AAV manufacturing and XLenti stable solutions for lentiviral manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHUwqHPDnhfMm8iJzwD6E--0a559J8xEuAa_fWKv2Km-51GlxlOIAUcsI1jgg0F762aVl3vX7Xl-JKDY2GiMXkVxsu_xuObCbkqd9TVc3i2UEa6V-T1FzJTOopwJm1fMkl66uGLqGoocM0=", "source": "WuXi AppTec Selected by IQVIA Stem Cell Center to Serve as GMP Manufacturer of Advanced Therapies", "page": "", "keywords": ["IQVIA Stem Cell Center", "GMP Manufacturer", "Advanced Therapies"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": null, "notes": "WuXi AppTec (parent company of WuXi Advanced Therapies) was selected by IQVIA Stem Cell Center as a GMP manufacturer of advanced therapies, indicating stem cell manufacturing capabilities."}]</t>
         </is>
       </c>
       <c r="F2" t="b">
@@ -567,37 +567,49 @@
       <c r="G2" t="n">
         <v>2</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>115.02</v>
+      </c>
+      <c r="I2" t="n">
+        <v>63.9</v>
+      </c>
       <c r="J2" t="n">
-        <v>110</v>
+        <v>89.45999999999999</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>127.8</v>
+      </c>
+      <c r="M2" t="n">
+        <v>91.29000000000001</v>
+      </c>
       <c r="N2" t="n">
-        <v>165</v>
+        <v>109.54</v>
       </c>
       <c r="O2" t="n">
         <v>2</v>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="P2" t="n">
+        <v>91.29000000000001</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>54.77</v>
+      </c>
       <c r="R2" t="n">
-        <v>18.33</v>
+        <v>73.03</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>183.33</v>
+        <v>182.57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "webSearchQueries": ["Takara Bio annual reports", "Takara Bio investor presentations", "Takara Bio earnings releases", "Takara Bio regulatory filings", "Takara Bio manufacturing sites", "Takara Bio advanced therapy CDMO", "Takara Bio CDMO revenue", "Takara Bio gene therapy manufacturing revenue", "Takara Bio stem cell manufacturing revenue", "Takara Bio AAV LV manufacturing"]}</t>
+          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "groundingChunks": [{"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHhZKK2q2bBMUBc3mEjYRdpYSezNoIhrB8SNhnL2PVweWiEJaAL-bEomIr_Kp3e2hzpo7K_ecWbV-G-zXA0hqGiOLoWx1qhLaluOaCs2RMXHslyq1v4duzv7V2RreaxEhkn-sjmcm_7M1H_3yhBd_KqFdiPhvAo0tY34kfCTpuyfHq7L0wzI5HJXiUuJB1NvT0wMbGFKyn6ZxxaVYtNjD0z", "title": "takara-bio.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFUdojeMlmtFgHD1bNwtofv9NzwInZu4_uRR_g2lurIC6ls_zcT0G7qmFAAMgpTn_34k58_jY8ojVpPk1PDZYrwTfs2PzdzyY53y10Fq33dvE0so3P39rUsfExQ7kJd0nlB4Y5eIXV_RY5QohRQDbbFcl4_y8Y=", "title": "takara-bio.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG3RjJNLbl3qsqnHjrlEiqqj3ShFQ_IbOcLdqYMYPWmu737pc0UqaC2BV8KSNyGYkSWVM32XWNW2tRmrHZxQfyiFJVwY6gzAS9h4nqMq7hD4GTo95HYDIPQn-sZU6thiK1dQ1XgHAGmz01BnFIQ", "title": "takara.co.jp"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFZVqij5GloB61FAeoAtyTA5AUT2SFWKGx-mhD2trVtU-DqCusg0FWZX4j3w7KWDxt18q5fj8C4BbmDKCMVL85b71DBTeQNg6v6B-_uIr7w4_bXnAGHoU3qkvWTghcw88v9kbsaVz3EKZQQLUq3ktkVIa51RK8=", "title": "xe.com"}}], "groundingSupports": [{"segment": {"startIndex": 14970, "endIndex": 15970, "text": "This is the primary source for advanced therapy manufacturing revenue.\"\n},\n{\n\"url\": \"https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFZVqij5GloB61FAeoAtyTA5AUT2SFWKGx-mhD2trVtU-DqCusg0FWZX4j3w7KWDxt18q5fj8C4BbmDKCMVL85b71DBTeQNg6v6B-_uIr7w4_bXnAGHoU3qkvWTghcw88v9kbsaVz3EKZQQLUq3ktkVIa51RK8=\",\n\"source\": \"Xe.com\",\n\"page\": \"Historical Rates Tables - JPY\",\n\"keywords\": [\"JPY to USD\", \"exchange rate\", \"March 31, 2024\"],\n\"bucket\": \"\",\n\"confidence\": 3,\n\"reported_or_inferred\": \"reported\",\n\"estimated_revenue\": {\n\"value\": null,\n\"range_low\": null,\n\"range_high\": null\n},\n\"notes\": \"Provides the JPY to USD exchange rate of 0.006608059156086096 on March 31, 2024, used for currency conversion.\"\n}\n],\n\"assumptions\": [\n\"The 'CDMO' segment revenue (¥7,997 million for FY2024) is considered the primary source for advanced therapy manufacturing revenue, as company descriptions consistently link CDMO to gene and cell therapy, viral vectors, and regenerative medicine manufacturing services."}, "groundingChunkIndices": [0, 1, 2]}, {"segment": {"startIndex": 15970, "endIndex": 16234, "text": "\",\n\"The 'Gene Therapy' segment revenue (¥2,653 million for FY2024) is excluded from advanced therapy manufacturing estimates as it appears to primarily relate to Takara Bio's own gene therapy product development and royalties, not contract manufacturing services."}, "groundingChunkIndices": [0]}, {"segment": {"startIndex": 16234, "endIndex": 16455, "text": "\",\n\"The 'Regenerative medicine' segment revenue (¥4,060 million for FY2024) is excluded as a separate total to avoid double-counting, as stem cell manufacturing is considered a component within the broader CDMO services."}, "groundingChunkIndices": [0]}, {"segment": {"startIndex": 16455, "endIndex": 16573, "text": "\",\n\"The JPY to USD exchange rate of 0.006608 USD/JPY as of March 31, 2024, was used to convert all JPY figures to USD."}, "groundingChunkIndices": [3]}], "webSearchQueries": ["Takara Bio investor relations", "Takara Bio annual report", "Takara Bio financial statements", "Takara Bio CDMO services", "Takara Bio gene therapy manufacturing", "Takara Bio viral vector manufacturing", "Takara Bio stem cell manufacturing", "Takara Bio advanced therapy manufacturing", "Takara Bio regenerative medicine CDMO", "Takara Bio GMP manufacturing", "Takara Bio Consolidated Financial Results for the Fiscal Year Ended March 31, 2024", "Takara Bio Annual Report 2024", "Takara Bio CDMO revenue 2024", "Takara Bio gene therapy revenue 2024", "Takara Bio stem cell revenue 2024", "JPY to USD exchange rate March 31 2024"]}</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -607,7 +619,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>["Takara Bio's total net sales for FY2025 (ended March 31, 2025) were \u00a545,039 million, which converts to approximately $295.33 million USD using an exchange rate of 1 USD = 152.5 JPY.", "The 'Gene Therapy' business segment, which includes advanced therapy CDMO services, is estimated to contribute 15-25% of Takara Bio's total net sales for FY2025. This is inferred from statements indicating that the 'Bioindustry' segment is the 'vast majority' of revenue, while the 'Gene Therapy' segment sales increased and the CDMO business as a whole saw a slight increase.", "Within the estimated Gene Therapy segment's manufacturing revenue, 60-70% is attributed to AAV/LV Viral Vector Manufacturing. This is based on explicit mentions of 'vector manufacturing' revenue increases and significant investments in 'viral vector manufacturing' capabilities.", "Within the estimated Gene Therapy segment's manufacturing revenue, 10-20% is attributed to Stem Cell Therapeutic Manufacturing. This considers the reported 'significant decline in cell processing revenues' in FY2025 but acknowledges the presence of 'GMP stem cell facilities' and 'iPSC manufacturing' activities.", "The remaining 10-30% of the estimated Gene Therapy segment's manufacturing revenue is attributed to other gene therapy manufacturing modalities (e.g., plasmid vector and mRNA production) that are not specifically AAV/LV or Stem Cell. This is based on the explicit mention of 'plasmid vector and mRNA production' as part of their CMO services."]</t>
+          <t>["The 'CDMO' segment revenue (\u00a57,997 million for FY2024) is considered the primary source for advanced therapy manufacturing revenue, as company descriptions consistently link CDMO to gene and cell therapy, viral vectors, and regenerative medicine manufacturing services.", "The 'Gene Therapy' segment revenue (\u00a52,653 million for FY2024) is excluded from advanced therapy manufacturing estimates as it appears to primarily relate to Takara Bio's own gene therapy product development and royalties, not contract manufacturing services.", "The 'Regenerative medicine' segment revenue (\u00a54,060 million for FY2024) is excluded as a separate total to avoid double-counting, as stem cell manufacturing is considered a component within the broader CDMO services.", "The JPY to USD exchange rate of 0.006608 USD/JPY as of March 31, 2024, was used to convert all JPY figures to USD.", "Stem Cell Therapeutic Manufacturing revenue is estimated to be 19-28% of the total CDMO revenue, reflecting Takara Bio's explicit GMP license for hES cell derivation and banking and expertise in cell processing. This translates to a range of $10.00 million to $15.00 million. (Inferred by segment apportionment based on qualitative evidence).", "Gene Therapy Manufacturing (broader, including AAV/LV) revenue is the remainder of the CDMO revenue after deducting the estimated Stem Cell Therapeutic Manufacturing revenue. This results in a range of $37.85 million to $42.85 million.", "AAV/LV Viral Vector Manufacturing revenue is estimated to be 60-75% of the total Gene Therapy Manufacturing revenue (within CDMO), given the strong emphasis on AAV and lentiviral vector manufacturing capabilities and large-scale production. This translates to a range of $22.71 million to $32.13 million. (Inferred by segment apportionment based on qualitative evidence).", "The 'value' for each bucket is the midpoint of its estimated range. The 'total_advanced_therapy_revenue' value is the reported CDMO revenue, and its range is the sum of the low and high ranges of the individual advanced therapy buckets."]</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -617,7 +629,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[{"source": "Clinical-grade viral vector production - Takara Bio", "page": "Overview", "keywords": ["viral vector production", "adeno-associated viral (AAV)", "lentiviral", "GMP guidelines", "small- and large-scale viral vector manufacturing"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Direct evidence of GMP manufacturing services for AAV and lentiviral vectors."}, {"source": "Research-grade viral vector production - Takara Bio", "page": "Gene and cell therapy manufacturing services", "keywords": ["research/preclinical-grade virus production services for: Retrovirus; Lentivirus; Adeno-associated virus (AAV)", "smooth transition to clinical-grade manufacturing", "scale-up development for future commercial manufacturing"], "bucket": "aav_lv", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Supports AAV/LV manufacturing capabilities with a pathway to clinical-grade production."}, {"source": "Cell and gene therapy manufacturing services - Takara Bio", "page": "Custom services", "keywords": ["manufacturing and quality-testing services for cellular and gene therapy products", "CMO services include plasmid vector and mRNA production, viral vector production, T-cell processing, cell banking, and quality testing", "State-of-the-art GMP manufacturing sites"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Broad CDMO services for cell and gene therapy, including viral vector and plasmid/mRNA production, and T-cell processing."}, {"source": "Advanced Therapy Medicinal Products CDMO Industry is Rising Rapidly - BioSpace", "page": "March 28 2024", "keywords": ["Takara Bio, Inc. launched CDMO Cell Therapy for gene therapy products using siTCR technology for its genetically modified T-cell therapy products."], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Confirms CDMO launch specifically for gene therapy products."}, {"source": "Takara Bio Group | TAKARA HOLDINGS INC.", "page": "Contract Development and Manufacturing Organization (CDMO)", "keywords": ["CDMO services for cutting-edge regenerative medicine products", "contract services for biologics development and manufacturing", "Center for Gene and Cell Processing (CGCP), is a large-scale one-stop center for development, manufacturing, and quality testing of gene therapy products."], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Explicitly states CDMO services for regenerative medicine and gene therapy, with a dedicated large-scale facility."}, {"source": "About Takara Bio", "page": "About Takara Bio", "keywords": ["GMP manufacturing site in West Japan\u2014the first of its kind\u2014enables seamless and sterile handling of viruses, cells, and proteins.", "GMP stem cell facilities in G\u00f6teborg, Sweden"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Confirms dedicated GMP facilities for stem cell manufacturing."}, {"source": "Takara Bio Establishes Foothold in the Pluripotent Stem Cell Market - BioInformant", "page": "Takara Bio's Cell and Gene Therapy CDMO Business", "keywords": ["contract manufacturing service for customers who are focused on clinical cell therapy applications", "human iPS and ES donor lines"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Strong evidence for stem cell contract manufacturing services and iPS/ES cell lines."}, {"source": "Consolidated Financial Results for the Fiscal Year Ended March 31, 2025 - Takara Bio Inc.", "page": "Page 13", "keywords": ["higher revenues from vector manufacturing, including mRNA vaccine related manufacturing", "significant decline in cell processing revenues", "CDMO business as a whole was a slight increase in revenues", "Takara Bio is in charge of the development and manufacturing of a AAV gene therapy drug"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Indicates growth in vector manufacturing (including AAV) and decline in cell processing within the CDMO business for FY2025. Also direct involvement in AAV gene therapy drug manufacturing."}, {"source": "What is Growth Strategy and Future Prospects of Takara Bio Company? - Matrix BCG", "page": "April 13 2026", "keywords": ["expanded Center for Gene and Cell Therapy in Shiga marks its shift from reagent supplier to global clinical-stage CDMO, leveraging decades of enzyme and PCR expertise to support advanced therapeutics", "upgraded its San Jose site to add high-throughput viral vector manufacturing", "Patented AAV purification achieves higher purity"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Reinforces CDMO focus on advanced therapeutics and specific expansion of viral vector (including AAV) manufacturing capabilities."}, {"source": "What is Brief History of Takara Bio Company? - Matrix BCG", "page": "April 13 2026", "keywords": ["ongoing expansion of Kusatsu and automation investments aim to scale viral vector and iPSC manufacturing"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Confirms manufacturing scale-up for iPSC, a type of stem cell."}]</t>
+          <t>[{"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFXnMTuV4nGwrD0UkTGP57dtyFbq_XCHoMhhcuBsubEufyPs2DsZFujb1oW5uwLnymkWQ5AIOcOkukr-9EXPYP_ybW3BDz_rucEZoCgVZdMgU6d2lTYmVGkCDui4wVC71eUAl4Nx-qDxwWb7ufg54fnkRv8nmvz2MoS5p8piI8sDXERmzN6HgnP63auHMKyhiGAoiKY_vUqsLZhNN94AzdSc5XhotvMyXmU_HP2a3JPjgpmB03yM362KdVYrg-loK9H6AaHcGJI", "source": "Takara Bio Website", "page": "Research-grade viral vector production", "keywords": ["AAV", "lentivirus", "viral vector", "production", "scale-up", "commercial manufacturing"], "bucket": "aav_lv", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Explicitly states offering research-grade AAV and lentivirus production services with scale-up development for future commercial manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEby0_ix8EeeIwXQO7c-jOMwx9AQLQPIXi1L-RcgBQNHbZAFDFmoBQBg-0nyyD27W2ABDiHQ5dTp3KwSLFtP-a-sEX30SxHSMPuSAVEae6dAENU6PuKEAHN4wK-vbZAx6kkJNt1WJ9TbS3X8EDasfsBrY4x_o9TIo8vehHMM1JKnHnYMl7A5KNAxPUoUgA=", "source": "Takara Bio Website", "page": "Cell and gene therapy manufacturing services", "keywords": ["CMO services", "viral vector production", "T-cell processing", "cell banking", "GMP manufacturing sites", "cellular and gene therapy products"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights comprehensive manufacturing and quality-testing services for cellular and gene therapy products, including viral vector production and cell banking, at GMP sites in Japan and Europe."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF6zNDZyKuzxygTRl8p3J66bE4ukE3UeiVGrTcZDglk-_11q-OktdT5asCLHcHFpUx1EPHUwagY-ETdNQgEySWwKQ-telHbt61J5BgJeG5ehj2rV65VSuJrV4rfgTMbtw==", "source": "BioInformant", "page": "Takara Bio Establishes Foothold in the Pluripotent Stem Cell Market", "keywords": ["cell and gene therapy manufacturing", "CDMO business", "Center for Gene and Cell Processing", "hES cells", "GMP conditions", "contract manufacturing service", "clinical cell therapy applications"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Details Takara Bio's CDMO business for cell and gene therapy, specifically mentioning a manufacturing license for derivation and banking of human embryonic stem (hES) cells under GMP conditions in Sweden as a contract manufacturing service for clinical cell therapy applications."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHOpk8nTAeaQFjrfZgFd-Ka0rsM-4lkqVL4JA1lskxJjfL2Hi5qWUMuGDETEQzY84zn3INLTWcav6PMDEHBfmRrVBsfwRKZnFQB6DQOYFC9QQuL_T_FyGvbyLRkijnmP2yuUm6vT7ZLcDCh615kpgE65HhsU6-9qeKrDR-KQQC2RmE_twjhUEpJ45CPUdvFEmqhNmJDI5wYn_rfCG4kAd2BzjVsR0vXY3c4UVIClXytDc8wpNpIKjPiZgiZCFRm2d9QoorVoHHYYuTeNvWC3Nxn", "source": "BioPharma APAC", "page": "Takara Bio Inc. Launches Large-Scale Viral Vector Manufacturing with Thermo Fisher's DynaDrive Bioreactors", "keywords": ["large-scale viral vector contract manufacturing", "CDMO", "gene and cell therapy", "GMP facilities"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Announces Takara Bio's launch of large-scale viral vector contract manufacturing using Thermo Fisher's DynaDrive Bioreactors, supporting gene and cell therapy development in GMP facilities."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHBWFYIvJA6sUXSR9f1dZD8yAn1xEsBZLWegRz58kcBxN1ARvbWAbDaFIWmabgYfkRQ5jPcX3vLt8V2dugnqOPoumDwPlYUf_9wb6mKQgbN831VI5uPiR_Gbe57gxpCYTpzMFmu3lsfQ1PwVeVetjLlbZHFMbZRaMfrzJXHwTF0EbKGM7zFR8Q8sDDFdr3P0Byo3jLytkzsa_5MBdFeMtBUr7Z96W0jOFzaF3uKRXVD5eQmff0wZk94So9Ku3vnZ1GWy9GQ5JZhtFi", "source": "Takara Bio USA News Release", "page": "Takara Bio expands GMP facility to accommodate a variety of modalities and strengthen supply chain", "keywords": ["GMP facility expansion", "viral vector production", "cell processing", "clinical-grade human embryonic stem cell line derivation", "gene and cell therapy manufacturing services", "regenerative medicines"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Describes the expansion of their Center for Gene and Cell Processing (CGCP) GMP facility to increase production capacity for gene therapy, cancer immunotherapy drugs, and regenerative medicines, including viral vector production and cell processing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEW7lUWweNDKeSgExFtgGr3M5Jqjp1bAZU5T_hBa970o7eOkDYJmWwoIzbzs2HG9Xo6V5O97OZkQ0ryKyYRJolxn2rtEy7VE8lAbDy_JEu13nHDKQtV5uvt4hedusaqAZwZ8Lrz-H1Vqoz5mC3VSnda6FbHXn_29ibB2osRCXY1cK1Zl6-v-48kEKmXzR5vUhwh2NoyEDX3iEMy4Vbcr6mxPkB5v8BFpQrV-3ibiEeKuWfrBw_PxsPodbE9c8u3", "source": "Takara Bio Website", "page": "Clinical-grade viral vector production", "keywords": ["virus production services", "AAV", "lentiviral", "retroviral vectors", "GMP manufacturing facility", "large-scale manufacturing"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights clinical-grade viral vector production services for AAV and lentiviral vectors, emphasizing their one-stop GMP manufacturing facility with capabilities up to 2,000 L."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG06PgLIRc0ScBbMWsuKwoV27crfweBb5CpLilYNGaQEIVpMRkMspgvATI88WPC0LjgjUT4KhvmSo9qt8USK447UE2Jj5yaRXR-96lEc4NvVKzxaHqDuCaSA8rMwMm3lqFYKg2QDMeF_NOaCjjHAwcs-UZjTyTdW_1JHQZRjt5NeryWH_pf0Gfwzqmj_EfFqARczULEaoQR", "source": "Takara Bio Website", "page": "Gene and cell therapy manufacturing services", "keywords": ["regenerative medicine development", "gene and cell therapy development process", "viral vector production", "cell banking", "genetically modified cell manufacturing", "cell processing", "GMP manufacturing facilities"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Offers support for regenerative medicine development and gene/cell therapy projects, including viral vector production, cell banking, and cell processing at GMP facilities."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFIEMC4p6wCz419z9p7B7E6MThJD95r6QqJmd8hdcLElO10ehp61vB6GtdH4JZiklXfE8jscsuk1b0k8mKwRjCgzblaywylTO5FbkvmSXRJJWMSQjJzTvSsvdH9IbKIiwyOM3FNZFeV39ypu88S_v13WSvN47sH_lCD", "source": "Takara Holdings Inc. Website", "page": "Takara Bio Group | Business", "keywords": ["CDMO business", "regenerative medicine products", "gene therapy products", "Center for Gene and Cell Processing (CGCP)", "viral vectors", "transduced cells"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "States that their CDMO business provides contract services for biologics development and manufacturing, focusing on regenerative medicine products and gene therapy products, and enhancing capabilities for viral vectors and transduced cells at CGCP."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHGjeE6IGfN7tXZ5Dd2b1BOlXFks0i9wrk7UJV6FnCo2t174QI6TNDyTFrwHiVR3ilHrJpxxCAHRD3eTAGLaPQRswLqYj9oxZtyD61HKhZipSai5ZSqmx6PZmlXoDIVThEr2roatglbSURQaYpKe38IXsC0PQ==", "source": "Takara Bio Inc. Website", "page": "AAV | Technologies / Projects | Gene Therapy", "keywords": ["AAV vectors", "contract manufacturing services", "CDMO services"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Explicitly states providing contract manufacturing services for various viral vectors, including AAV vectors, and CDMO services for CereAAV\u2122 series."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEds-lmFxvQffiLmHCw7F-HOcC1j4GPcbMkDZ98uGpyMtsGg-X77A0iYtcvqbKNaRH3VxD5Z1U83S0tOKyHeoEO-92gZlm_QMm66LKllbRlZrvW2jE_Zdt1XER4zGaN219FZ0kN1z4nrDkxNLVEKQAvAQ==", "source": "Matrix BCG", "page": "What is Growth Strategy and Future Prospects of Takara Bio Company?", "keywords": ["CDMO", "viral vector manufacturing", "gene and cell therapy market", "regenerative medicine"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Mentions Takara Bio's shift to a global clinical-stage CDMO supporting advanced therapeutics, including high-throughput viral vector manufacturing and services for regenerative medicine."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHSHW5euDjoxBvXvHNFhpr4MNf7cj3c1q7n1XgtAdt11xVEELOQt8-g8LYD3KykSK6mXZnPq_yqlXwBKb0hHxTa1WBwDyybGapUX4g1cABEyHWNXR_0GF2lmF33SdJiovWN_0PlzXl5ctBwpnE-v69m-xnsb-A5McqvATll_h8UpnrwnJeMlYVnNZ8cShgzitix236FxHhBhff3U8We7EL__MPIDNv1LAk3L6zgc8M6UKb-4d1H6AM-s10Co4LVUAWv7ET0tqS-2J4jnjSkvQCoRhUX2kMILNwVhiPODAfCk7YlQNuS39T9R1bk29VcIfb_ZtL_0P3nIqxTpvt3YXKkMAWYxLTp0ep4Z17ZWA==", "source": "PR Newswire", "page": "Takara Bio granted manufacturing license from the Swedish Medical Product Agency for clinical-grade human embryonic stem cell line derivation and banking", "keywords": ["manufacturing license", "hES cells", "GMP conditions", "contract manufacturing service", "gene and cellular therapy industries"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Reports on Takara Bio receiving a manufacturing license for clinical-grade human embryonic stem cell line derivation and banking under GMP conditions in Sweden, offered as a contract manufacturing service."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHYTsQnjfj9XkkS0CfcBa5V3_JyN0W6AmVwTmxh_N3qJ3DJaVXvfUzWia1953REuRXppd5WPHPqd8sAT14HpoIU6-0V_Bso0WPTVGeL1lcqwEKMMwEPzNeMGp_gcEMKq0Pzu4kZX25Q61hBZAqZFF5n8FDGcVh0ZShoM2oXYzJGnbcxn4xfYEtDxAufvm1JJ_fgC6lkdkycy0siM4p-WU_T4C6oapW6UVihRVbIkk1l-sjXyw==", "source": "Takara Bio Website", "page": "GMP-grade plasmid production", "keywords": ["GMP-grade plasmid production", "gene therapy products", "Master Cell Bank", "bioreactor"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Describes GMP-grade plasmid DNA production services for gene therapy products, including MCB preparation and large-scale bioreactor production, which is a critical component for viral vector manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEeI0g5-nTC8--Yq0Ry89EslEAIj_BTg8YH-gB2kd4yRwWzJS2qMk1qgtcioydUCbj7lCOjWqtk1-b8bt340iRcvezb0o6LvrxH_Rl2eVtBYAfvA_vGZ1K8kzohnJIS6jSasiysjl4oqJLvDA==", "source": "Takara Bio Inc. Website", "page": "CDMO | Business", "keywords": ["CDMO", "biologics development and manufacturing", "regenerative medicine products", "viral vectors", "transduced cells"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Defines their CDMO business as providing contract services for biologics development and manufacturing, with a focus on regenerative medicine products and enhancing capabilities for viral vectors and transduced cells."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHBWFYIvJA6sUXSR9f1dZD8yAn1xEsBZLWegRz58kcBxN1ARvbWAbDaFIWmabgYfkRQ5jPcX3vLt8V2dugnqOPoumDwPlYUf_9wb6mKQgbN831VI5uPiR_Gbe57gxpCYTpzMFmu3lsfQ1PwVeVetjLlbZHFMbZRaMfrzJXHwTF0EbKGM7zFR8Q8sDDFdr3P0Byo3jLytkzsa_5MBdFeMtBUr7Z96W0jOFzaF3uKRXVD5eQmff0wZk94So9Ku3vnZ1GWy9GQ5JZhtFi", "source": "Takara Bio USA News Release", "page": "Takara Bio expands GMP facility to accommodate a variety of modalities and strengthen supply chain", "keywords": ["GMP manufacturing facilities", "viral vector production", "cell processing", "clinical-grade human embryonic stem cell line derivation", "quality testing", "cell banking"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Mentions services for clinical-grade human embryonic stem cell line derivation, cell processing, and cell banking at their GMP facilities."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEZXkljXmHqLgjL0OMHD8aWIuZluNkOYEtJjUztQOkubnWX0KwSwcHoBCK_ufWw3dYUaTmzUfjK_IJHSxa3bQ6Cpagx1CDdw-eDtvlc38SAXa3pZNdi28JKgonWlj5Inaa-4Xm0qi8q7FGTtfmvkwHb2rKyEOeCFbxUE4K56jE93YrsvKlREF-3tThvHnmAqMz9WEIsKJM=", "source": "Takara Bio Website", "page": "CMO services", "keywords": ["T-cell processing", "Mesenchymal stem cells", "gene and cell therapy products"], "bucket": "stem_cell", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lists expertise in T cells, NK cells, and Mesenchymal stem cells as part of their T-cell processing service for gene and cell therapy products."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHhZKK2q2bBMUBc3mEjYRdpYSezNoIhrB8SNhnL2PVweWiEJaAL-bEomIr_Kp3e2hzpo7K_ecWbV-G-zXA0hqGiOLoWx1qhLaluOaCs2RMXHslyq1v4duzv7V2RreaxEhkn-sjmcm_7M1H_3yhBd_KqFdiPhvAo0tY34kfCTpuyfHq7L0wzI5HJXiUuJB1NvT0wMbGFKyn6ZxxaVYtNjD0z", "source": "Takara Bio Inc. Financial Results Presentation", "page": "Consolidated Financial Results for the Fiscal Year Ended March 31, 2024", "keywords": ["CDMO", "7,997", "million yen"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 52.85, "range_low": null, "range_high": null}, "notes": "Reports CDMO segment net sales of \u00a57,997 million for the fiscal year ended March 31, 2024. This is the primary source for advanced therapy manufacturing revenue."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFZVqij5GloB61FAeoAtyTA5AUT2SFWKGx-mhD2trVtU-DqCusg0FWZX4j3w7KWDxt18q5fj8C4BbmDKCMVL85b71DBTeQNg6v6B-_uIr7w4_bXnAGHoU3qkvWTghcw88v9kbsaVz3EKZQQLUq3ktkVIa51RK8=", "source": "Xe.com", "page": "Historical Rates Tables - JPY", "keywords": ["JPY to USD", "exchange rate", "March 31, 2024"], "bucket": "", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Provides the JPY to USD exchange rate of 0.006608059156086096 on March 31, 2024, used for currency conversion."}]</t>
         </is>
       </c>
       <c r="F3" t="b">
@@ -627,52 +639,52 @@
         <v>2</v>
       </c>
       <c r="H3" t="n">
-        <v>51.68</v>
+        <v>32.13</v>
       </c>
       <c r="I3" t="n">
-        <v>26.58</v>
+        <v>22.71</v>
       </c>
       <c r="J3" t="n">
-        <v>39.13</v>
+        <v>27.42</v>
       </c>
       <c r="K3" t="n">
         <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>22.15</v>
+        <v>42.85</v>
       </c>
       <c r="M3" t="n">
-        <v>4.43</v>
+        <v>37.85</v>
       </c>
       <c r="N3" t="n">
-        <v>13.29</v>
+        <v>40.35</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="n">
-        <v>14.77</v>
+        <v>15</v>
       </c>
       <c r="Q3" t="n">
-        <v>4.43</v>
+        <v>10</v>
       </c>
       <c r="R3" t="n">
-        <v>9.6</v>
+        <v>12.5</v>
       </c>
       <c r="S3" t="n">
-        <v>88.59999999999999</v>
+        <v>57.85</v>
       </c>
       <c r="T3" t="n">
-        <v>35.44</v>
+        <v>47.85</v>
       </c>
       <c r="U3" t="n">
-        <v>62.02</v>
+        <v>52.85</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "groundingChunks": [{"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFEYdzzuI5ni6sZ7XzQ2vn1Dh1Jm81f7ABtCvxr5IBV_OcXLfU64krM4nyumz0E4OqWKOvhlxvSPOew3zftbHfCyvgkK_uos0OOwdK0XBYIdol4xqia4xwtkzvJZKjSsdf88nUogHoFVC4cFNEn4GuCcA==", "title": "lonza.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHirF9uh-eOjuIOcjgwbap5KKZdSJqPTmY5E6ksy7-yQQ56VX28-QU39b6z1yMnqXSa1XynDUVY7OQWQuIUAegJiRBCXSSoqxN-2zFoHeohc2pLbaX3uuUxH4nX54-uhL9Nih2hQAm20YnzYBEycqxbK_rYCYit6SeG7mMNOI0r_h5Y29_iMSi8", "title": "lonza.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH9U-nuSZ4Cudw1V1PKzKsJZJyL2funsZgQdkwCdgJMHo1ldSBMm3XMNyuCD1A1aUDGj-0UkQFCZEz4oCwsWyDH24ZY3h_1-nY5BRCZE99wYAiZ60RdloVDQzi5FGQ5iS68-QAAkxGK1D8-gwohsHyptURuSrQVolgzFRjZ01m4MyWj5g==", "title": "lonza.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEsZdMr-3Itg3zwid6Y-9io71cN-Lztr_ehO7p9uZiwXyQBBq_3ND1LT095cLIwE_IiahFEqCxq28dhQaWV9g9wvJhljkN40fgr73sdr1Ak4xXJg8TEWyqlWnpDfT2N2YI0bK8QF4gaUaFR8LBArCuyMLkIsm5PqMBf5rnUtRc8_T2kiZfFUa_urPSalisy4w==", "title": "lonza.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFB3ITf_LWHDDH_uu-FBJ6wXlQ3GduUaHS3TSWPxrqlL41yJjAcuNfemRy3scAGIsCXj6vwUIpI5mqEerBC2XoUhPM3A9i9KoQRp6lnoayML931uQLVaWST3_eS17Kq565GHRmtvZiuYsLEvSCDpB3bb4W1lsszhrtVVEc=", "title": "lonza.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFXH5n3MKQt4LgrVkXvqgv0R5363lIDrCguaguRC8Tj7iXpLsIushJ7363ChB8CssMTn4LE1KHiSd5vGI5D46XG2LRmI_oGgJYOqXJQfjMgiGpHd19rYh1ILCUHVHVzAUuCFB8s5U8GNy8mNNUImg7BMC6WCNhpSkcvGPdoTKpCghMBjvP8Yj9UAEWZN1g=", "title": "grandviewresearch.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFLDOVHrqvd0oaQxgF1oTXduQDHNGT-smj5jGoYACrh53DDH_tEUtB-CCrVW-fkoKXnkS9GxDyl7IudKeuNjKtUledVOLwFILaQy10qI51VsSgmgpi5-SkT1m0CD5R86b5dc5PH_E7kGdFVJ3THay_ccyUrOQIs9EKqNVK2N1Ad2nYs6TMtuCWdWa7ceOcnf6W0qLtTKoYZ6w==", "title": "lonza.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGcsKbNl2i14QCvnuZsflTTthMsgAToGLj71WMJYuBZr5-OabdxhbeeP0Vwrv8tzUyNe_9B4M3lhrdX6pNob8Xr4-HfPvZADQjtsM4S7PstVSlrN6aAesCJGfCbs1D8w33NE5a2mPSKJQfs2QyjFOk4JQjFl4eQmldbCdBnaEZO5ZjpmVa40TleGUfZIGu6npubZQ==", "title": "strategicmarketresearch.com"}}], "groundingSupports": [{"segment": {"endIndex": 1056, "text": "```json\n{\n\"company\": \"Lonza Group (APAC Viral Div.)\",\n\"summary\": {\n\"aav_lv_revenue_estimate\": {\n\"value\": null,\n\"range_low\": 40.59,\n\"range_high\": 81.18,\n\"confidence\": 1\n},\n\"gene_therapy_revenue_estimate\": {\n\"value\": null,\n\"range_low\": 40.59,\n\"range_high\": 81.18,\n\"confidence\": 1\n},\n\"stem_cell_revenue_estimate\": {\n\"value\": null,\n\"range_low\": 20.0,\n\"range_high\": 50.0,\n\"confidence\": 1\n},\n\"total_advanced_therapy_revenue\": {\n\"value\": null,\n\"range_low\": 60.59,\n\"range_high\": 131.18\n}\n},\n\"evidence\": [\n{\n\"source\": \"Lonza Website - Singapore\",\n\"page\": \"Tuas site description\",\n\"keywords\": [\"allogeneic cell therapy products\", \"center of excellence for allogeneic cell therapy\", \"cGMP production\"],\n\"bucket\": \"stem_cell\",\n\"confidence\": 3,\n\"reported_or_inferred\": \"inferred\",\n\"estimated_revenue\": {\n\"value\": null,\n\"range_low\": 20.0,\n\"range_high\": 50.0\n},\n\"notes\": \"Lonza's Tuas site in Singapore is a CDMO facility designated for the contract development and production of allogeneic cell therapy products and is a center of excellence for allogeneic cell therapy."}, "groundingChunkIndices": [0]}, {"segment": {"startIndex": 1056, "endIndex": 1655, "text": "\"\n},\n{\n\"source\": \"Lonza Website - cGMP Manufacturing for Cell &amp; Gene Therapies\",\n\"page\": \"Capabilities section\",\n\"keywords\": [\"viral vector gene therapy\", \"cGMP manufacturing capabilities\", \"Singapore\", \"Asia\", \"allogeneic cell therapies\"],\n\"bucket\": \"gene_therapy\",\n\"confidence\": 3,\n\"reported_or_inferred\": \"inferred\",\n\"estimated_revenue\": {\n\"value\": null,\n\"range_low\": 40.59,\n\"range_high\": 81.18\n},\n\"notes\": \"Lonza's cGMP manufacturing capabilities span autologous and allogeneic cell therapies and viral vector gene therapy, with sites spread across the US, Europe, and Asia, including Singapore."}, "groundingChunkIndices": [1]}, {"segment": {"startIndex": 1655, "endIndex": 2293, "text": "\"\n},\n{\n\"source\": \"Lonza Website - Viral Vectors Manufacturing Services (CDMO)\",\n\"page\": \"Overview\",\n\"keywords\": [\"AAV\", \"lentivirus\", \"viral vectors\", \"development, clinical and commercial manufacturing\", \"GMP production\", \"suspension-based processes\", \"2,000 L\"],\n\"bucket\": \"aav_lv\",\n\"confidence\": 2,\n\"reported_or_inferred\": \"inferred\",\n\"estimated_revenue\": {\n\"value\": null,\n\"range_low\": 40.59,\n\"range_high\": 81.18\n},\n\"notes\": \"Lonza has a long-standing history in the development, clinical, and commercial manufacturing of viral vectors, including AAV and lentivirus, offering suspension-based processes up to 2,000L for GMP production."}, "groundingChunkIndices": [2]}, {"segment": {"startIndex": 2293, "endIndex": 2892, "text": "\"\n},\n{\n\"source\": \"Lonza Annual Report 2024\",\n\"page\": \"Cell &amp; Gene section\",\n\"keywords\": [\"manufacture the viral vector, cell therapy or gene therapy for five commercial cell and gene therapy products in three continents: the United States, Europe and Asia\"],\n\"bucket\": \"gene_therapy\",\n\"confidence\": 2,\n\"reported_or_inferred\": \"inferred\",\n\"estimated_revenue\": {\n\"value\": null,\n\"range_low\": 40.59,\n\"range_high\": 81.18\n},\n\"notes\": \"As of 2024, Lonza manufactures the viral vector, cell therapy, or gene therapy for five commercial cell and gene therapy products across three continents, including Asia."}, "groundingChunkIndices": [3, 4]}, {"segment": {"startIndex": 2892, "endIndex": 3449, "text": "\"\n},\n{\n\"source\": \"Asia Pacific Viral Vector Market Size &amp; Outlook, 2026-2033\",\n\"page\": \"Highlights\",\n\"keywords\": [\"Asia Pacific viral vector market generated a revenue of USD 811.8 million in 2025\", \"Lonza Group Ltd\", \"Key market players worldwide\"],\n\"bucket\": \"aav_lv\",\n\"confidence\": 1,\n\"reported_or_inferred\": \"inferred\",\n\"estimated_revenue\": {\n\"value\": null,\n\"range_low\": 40.59,\n\"range_high\": 81.18\n},\n\"notes\": \"The Asia Pacific viral vector market generated a revenue of USD 811.8 million in 2025, with Lonza Group Ltd identified as a key market player."}, "groundingChunkIndices": [5]}, {"segment": {"startIndex": 3449, "endIndex": 4316, "text": "\"\n},\n{\n\"source\": \"Annual Report 2021\",\n\"page\": \"Expanding Clinical Development and Manufacturing in Asia\",\n\"keywords\": [\"Expanding Clinical Development and Manufacturing in Asia\", \"mammalian development services in Singapore\", \"Viral vector manufacturing for gene therapy including the production of adeno-associated virus (AAV), lentiviral and oncolytic viral vectors\", \"Induced Pluripotent Stem Cell (iPSC) manufacturing expertise\", \"Stem cell high-throughput large scale manufacturing\"],\n\"bucket\": \"gene_therapy\",\n\"confidence\": 2,\n\"reported_or_inferred\": \"inferred\",\n\"estimated_revenue\": {\n\"value\": null,\n\"range_low\": 40.59,\n\"range_high\": 81.18\n},\n\"notes\": \"Lonza expanded its mammalian development services in Singapore in 2021, and its capabilities include viral vector manufacturing for gene therapy (AAV, lentiviral) and iPSC/stem cell manufacturing expertise."}, "groundingChunkIndices": [6]}, {"segment": {"startIndex": 4674, "endIndex": 5074, "text": "' or a granular breakdown of Cell &amp; Gene Technologies revenue by region or specific modality within APAC, revenue estimates are inferred from broader market data and Lonza's confirmed operational presence and capabilities.\",\n\"The APAC viral vector market size of USD 811.8 million in 2025 is used as a benchmark for estimating Lonza's revenue from AAV/LV and gene therapy manufacturing in the region."}, "groundingChunkIndices": [5]}, {"segment": {"startIndex": 5074, "endIndex": 5226, "text": "\",\n\"Lonza's market share in the APAC viral vector market is conservatively estimated to be between 5% and 10%, given its status as a 'key market player'"}, "groundingChunkIndices": [5, 7]}, {"segment": {"startIndex": 5432, "endIndex": 5594, "text": "\",\n\"Revenue for Stem Cell Therapeutic Manufacturing in APAC is inferred based on Lonza's Singapore site being a 'center of excellence for allogeneic cell therapy'"}, "groundingChunkIndices": [0, 1]}], "webSearchQueries": ["Lonza Group APAC Viral Div.", "Lonza Group Asia Pacific viral vector manufacturing revenue", "Lonza Group annual report advanced therapy manufacturing", "Lonza Group investor presentation gene therapy revenue", "Lonza Group Singapore viral vector manufacturing", "Lonza Group Guangzhou viral vector manufacturing", "Lonza Group advanced therapy manufacturing sites APAC"]}</t>
+          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "groundingChunks": [{"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHdQ8Pzdtg1FGzbolCJiOL5RSuFSwTCPtswTCuZCpKsdJj7M3bDEqIEZBIdu_bw7EWNJd7243sYk_a1Ofmw-p-pVAWr_eM9pduDUwmWET7JdxFf66JVCGkCMo6Ziza4iteiLqzYTmvD7RLb_vP8tEGiFI-N3uCuG1CgjjNF92unHoWIjqcVBsdnPEHSs86788=", "title": "mordorintelligence.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHQaGjjLZjhzTrDjoI1IocJQCdaSnAgRjBGhL_PVFwK26Peu0A_KZy248MEOY505Rf2vpqufb2ZDrMHdLsaOFtwIVVU20qX_qbbe3KBnLnSz6dk7pR1M8AynNG61SNMbwulpH39DHoLEv9xUSw6hMmNaW7CABhdDFWghmAyDyxuI4qfINPUN95AYD0vxMrsBHYfqoV2lmcZE5rDHnfbgeAMF9PucPG22T_I6A==", "title": "fiercepharma.com"}}], "groundingSupports": [{"segment": {"startIndex": 19145, "endIndex": 19687, "text": "This is based on the number of Lonza's sites in Asia (6 out of 30+ global sites) and the reported 18% APAC revenue growth for Lonza's CDMO business in 2024.\",\n\"70-80% of Lonza's APAC CGT revenue is attributed to gene therapy manufacturing (including AAV/LV viral vectors), reflecting the strong market focus on these modalities.\",\n\"AAV/LV viral vector manufacturing is estimated to account for 72.18% of the gene therapy manufacturing revenue, based on the reported market share of AAV vectors in the viral vector manufacturing market in 2025"}, "groundingChunkIndices": [0]}, {"segment": {"startIndex": 19688, "endIndex": 20069, "text": "\",\n\"20-30% of Lonza's APAC CGT revenue is attributed to stem cell therapeutic manufacturing, as it is a distinct but related advanced therapy modality where Lonza has stated capabilities and a facility in Singapore.\",\n\"All revenue figures are converted from CHF to USD using an approximate exchange rate of 1 CHF = 1.102 USD, based on Lonza's reported 2024 sales in both currencies"}, "groundingChunkIndices": [1]}], "webSearchQueries": ["Lonza Group APAC Viral Div. revenue", "Lonza APAC viral vector manufacturing revenue", "Lonza Singapore viral vector manufacturing revenue", "Lonza advanced therapy manufacturing APAC revenue", "Lonza gene therapy manufacturing APAC revenue", "Lonza annual report advanced therapy manufacturing", "Lonza investor presentation advanced therapy manufacturing", "Lonza press release viral vector APAC", "Lonza cell and gene therapy manufacturing sites APAC"]}</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -682,7 +694,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>["Lonza Group (APAC Viral Div.) refers to Lonza's viral vector and advanced therapy manufacturing activities within the Asia Pacific region, primarily centered around its Singapore site, as a distinct financial reporting division is not publicly disclosed.", "Due to the absence of explicit revenue figures for Lonza's 'APAC Viral Div.' or a granular breakdown of Cell &amp; Gene Technologies revenue by region or specific modality within APAC, revenue estimates are inferred from broader market data and Lonza's confirmed operational presence and capabilities.", "The APAC viral vector market size of USD 811.8 million in 2025 is used as a benchmark for estimating Lonza's revenue from AAV/LV and gene therapy manufacturing in the region.", "Lonza's market share in the APAC viral vector market is conservatively estimated to be between 5% and 10%, given its status as a 'key market player' and the competitive landscape. This range is applied to both AAV/LV and the broader Gene Therapy category, as AAV/LV represents the primary identified gene therapy manufacturing activity for Lonza in APAC.", "Revenue for Stem Cell Therapeutic Manufacturing in APAC is inferred based on Lonza's Singapore site being a 'center of excellence for allogeneic cell therapy', suggesting significant operational activity. A range of USD 20-50 million is estimated as a plausible scale of operations relative to viral vector manufacturing, in the absence of specific market share data for APAC stem cell manufacturing."]</t>
+          <t>["Lonza Group (APAC Viral Div.) is not a separately reported entity. Revenue estimates are inferred based on Lonza's global Cell &amp; Gene Technologies (CGT) business and its known presence and activities in the APAC region.", "Lonza's CDMO revenue is estimated to be approximately 90% of its total reported sales in 2024 (USD 7.24 billion).", "Lonza's global Cell &amp; Gene Technologies (CGT) revenue is estimated to be 8-15% of its total CDMO revenue. This range accounts for varying performance descriptions in different reports (e.g., 'strong performance' in 2024 vs. 'softer performance' in 2023 and 2025).", "Lonza's APAC region is estimated to contribute 15-25% of its global CGT revenue. This is based on the number of Lonza's sites in Asia (6 out of 30+ global sites) and the reported 18% APAC revenue growth for Lonza's CDMO business in 2024.", "70-80% of Lonza's APAC CGT revenue is attributed to gene therapy manufacturing (including AAV/LV viral vectors), reflecting the strong market focus on these modalities.", "AAV/LV viral vector manufacturing is estimated to account for 72.18% of the gene therapy manufacturing revenue, based on the reported market share of AAV vectors in the viral vector manufacturing market in 2025.", "20-30% of Lonza's APAC CGT revenue is attributed to stem cell therapeutic manufacturing, as it is a distinct but related advanced therapy modality where Lonza has stated capabilities and a facility in Singapore.", "All revenue figures are converted from CHF to USD using an approximate exchange rate of 1 CHF = 1.102 USD, based on Lonza's reported 2024 sales in both currencies."]</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -692,7 +704,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[{"source": "Lonza Website - Singapore", "page": "Tuas site description", "keywords": ["allogeneic cell therapy products", "center of excellence for allogeneic cell therapy", "cGMP production"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 20.0, "range_high": 50.0}, "notes": "Lonza's Tuas site in Singapore is a CDMO facility designated for the contract development and production of allogeneic cell therapy products and is a center of excellence for allogeneic cell therapy."}, {"source": "Lonza Website - cGMP Manufacturing for Cell &amp; Gene Therapies", "page": "Capabilities section", "keywords": ["viral vector gene therapy", "cGMP manufacturing capabilities", "Singapore", "Asia", "allogeneic cell therapies"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 40.59, "range_high": 81.18}, "notes": "Lonza's cGMP manufacturing capabilities span autologous and allogeneic cell therapies and viral vector gene therapy, with sites spread across the US, Europe, and Asia, including Singapore."}, {"source": "Lonza Website - Viral Vectors Manufacturing Services (CDMO)", "page": "Overview", "keywords": ["AAV", "lentivirus", "viral vectors", "development, clinical and commercial manufacturing", "GMP production", "suspension-based processes", "2,000 L"], "bucket": "aav_lv", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 40.59, "range_high": 81.18}, "notes": "Lonza has a long-standing history in the development, clinical, and commercial manufacturing of viral vectors, including AAV and lentivirus, offering suspension-based processes up to 2,000L for GMP production."}, {"source": "Lonza Annual Report 2024", "page": "Cell &amp; Gene section", "keywords": ["manufacture the viral vector, cell therapy or gene therapy for five commercial cell and gene therapy products in three continents: the United States, Europe and Asia"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 40.59, "range_high": 81.18}, "notes": "As of 2024, Lonza manufactures the viral vector, cell therapy, or gene therapy for five commercial cell and gene therapy products across three continents, including Asia."}, {"source": "Asia Pacific Viral Vector Market Size &amp; Outlook, 2026-2033", "page": "Highlights", "keywords": ["Asia Pacific viral vector market generated a revenue of USD 811.8 million in 2025", "Lonza Group Ltd", "Key market players worldwide"], "bucket": "aav_lv", "confidence": 1, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 40.59, "range_high": 81.18}, "notes": "The Asia Pacific viral vector market generated a revenue of USD 811.8 million in 2025, with Lonza Group Ltd identified as a key market player."}, {"source": "Annual Report 2021", "page": "Expanding Clinical Development and Manufacturing in Asia", "keywords": ["Expanding Clinical Development and Manufacturing in Asia", "mammalian development services in Singapore", "Viral vector manufacturing for gene therapy including the production of adeno-associated virus (AAV), lentiviral and oncolytic viral vectors", "Induced Pluripotent Stem Cell (iPSC) manufacturing expertise", "Stem cell high-throughput large scale manufacturing"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 40.59, "range_high": 81.18}, "notes": "Lonza expanded its mammalian development services in Singapore in 2021, and its capabilities include viral vector manufacturing for gene therapy (AAV, lentiviral) and iPSC/stem cell manufacturing expertise."}]</t>
+          <t>[{"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF9gy3ZzPEFNDYDTf-rngR4XAjFxaBnYzGLJV2g73nLvw5tUGrq79rjPvO98uXEjZ4Gz4TUeDBuUcBDh4syrbv8ay6ModISOx2-fl7G0pKhXYpwarnbeF4QBYDtsjj4OyCu-S2Sy-xtoAc2t3xr69aHkIUCyqViOYj58uNLH0fWF0CNUsNVeEi31SIBPHxW3LQSLOaUNU8cVsffSV2pSw==", "source": "Our Businesses - Lonza", "page": "7", "keywords": ["Cell &amp; Gene Technologies", "manufacture", "viral vector", "cell therapy", "gene therapy", "Asia"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "States Lonza manufactures viral vector, cell therapy, or gene therapy for commercial products in Asia."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFeBbu9U35AL4cr_CqDF7l_6d717-Gb6cM40EarpEWdQcFMa0XdiMXTg3cxrTilh6fW3S30Zn_VwBrsEUS_SDYCe2CtyZqwW6d6JO_fK3uu1c2xBhV35J-7hDeNVQ34eMlVr8iJXEG7WeiJpynUdhAXg_KUF2FA7w9ebc=", "source": "Cell Gene - Lonza", "page": "", "keywords": ["Cell &amp; Gene Technologies", "CDMO", "cell and gene therapies", "Asia", "viral vector", "cell therapy", "gene therapy"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Confirms Lonza's Cell &amp; Gene Technologies business unit offers CDMO services for cell and gene therapies and has manufacturing presence in Asia."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGLemyx0i4cFwZgd74ZxordT8pUDmqoBubkdc4wZ0C-aMthUj4N2slSf8E0vHILyaG8ToCXEX-K8iTnu9UMYGKUR43SaGPhK0rx92Fcwr_iW2F4dMFqPbcmC2z_IB6PoH3Yrvk=", "source": "Lonza 2024 - Annual Report", "page": "", "keywords": ["Cell &amp; Gene Technologies", "manufacturing sites"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Mentions Lonza's global development and manufacturing sites, which include CGT."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGLemyx0i4cFwZgd74ZxordT8pUDmqoBubkdc4wZ0C-aMthUj4N2slSf8E0vHILyaG8ToCXEX-K8iTnu9UMYGKUR43SaGPhK0rx92Fcwr_iW2F4dMFqPbcmC2z_IB6PoH3Yrvk=", "source": "Lonza 2024 - Annual Report", "page": "", "keywords": ["CDMO", "sales"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lonza's total sales in 2024 were CHF 6.57 billion."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG3D5HiQ9AKA_ZcBEiK8AV9e0W8tX_4xOD1VtTOa9CqBgusNzvgd5pKPF2D5oz437mCHGqFsnVhvRYny9lc-lPhF2pGXhVrg8pfhm_NvWDr-TqUB-jSpbu6w5NgcGVkIPBiVa6-vErtG3-64RE=", "source": "Marketing Mix Analysis of Lonza Group \u2013 MatrixBCG.com", "page": "", "keywords": ["APAC revenue", "CDMO contracts", "Singapore", "China", "biologics clients"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "APAC revenue +18% in 2024; Localized manufacturing captured ~30% of Lonza's new APAC CDMO contracts in 2024. Lonza expanded facilities in China and Singapore."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEgJbpuNuWZ_5BW73pJr0S1EwaSnfXUxu4aAfDY8x2O6M6J5A8pRvuPC0BmR_3EZw7fgioT4DHMFLm1Bbx_-Y3656iUjGW63tln4QyUVtRxhqKHArXr0liIhGhHNMI6a7V_-tRZz7utFdjS9vehA5Genr190XBWqRE0ET0qAn90MmyixKNyoolJ", "source": "cGMP Manufacturing for Cell &amp; Gene Therapies - Lonza", "page": "", "keywords": ["cGMP manufacturing", "cell therapies", "viral vector gene therapy", "Asia"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lonza's cGMP manufacturing capabilities span cell therapies and viral vector gene therapy across three continents, including Asia."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQENsAChUB91eOtskP1Q5XQeHX9TauQ2JpJJ3THvO3qDxkbQa5BCRSeB97tgVbuSw7DyzhgN6JG8H0GZ90MWGLUMIetSvE8MEuWYgmcBbKiv6K2uxLEKDp357IvNIExr3TUAST-E1H0=", "source": "Lonza - Company Presentation - YouTube", "page": "", "keywords": ["cell therapy manufacturing", "R&amp;D", "process development", "manufacturing of cells", "Singapore"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "A 2013 presentation explicitly states Lonza has a facility in Singapore for cell therapy related R&amp;D, process development, and manufacturing of cells, including pluripotent stem cells."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGGnCv4RH-fV4xECqlVfhx1hEJcEVC2JhSc_32dmNNT933jj9Op4W-Q6Egu94Vulgv2cLbfM3pbxZ63KdMz_L6mhGJlGmiJPYKJhTOZMGoRnEyLqkvjnyhOhgPt3ckz0bW987OfSOcP", "source": "Locations Worldwide | Lonza", "page": "", "keywords": ["Singapore", "Nansha, China", "Asia", "manufacturing sites"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lists Singapore and Nansha, China as Lonza locations in Asia with manufacturing capabilities."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFq4eb1fAaz24IU77clMz71kwVLEZpqW0O36s6LkjrRgZlT19TkkzKBfFWAT_Qv3pOdf0dJrMrvM1zjWsniLiTj0OOB7Z3-rWi39jR9iqD7rLu33PryPZtq9tC---uHwmfOpHNtke8MzRXKgdryWx0kwq3FDamk9B7f2s7XgDnQ0keOr-4IWcaVWXhueoGA2WGuO9YbC4v455QsZtNnwYg4j8fQgtF2Ot1v0ljqWNTCPGxvBKOt5Uw_fCQ12BeUfDc266BqM_89za0O86z9JDsBKCd4orZIOTXqlc767qtqZ_wKaMDACUex_fCcm4TyRzk2nv0AoLWS6fb-nw==", "source": "Avalanche Biotechnologies, Inc. and Lonza Announce Global Manufacturing Collaboration for Adeno-associated Viral Vectors for Gene Therapy - PR Newswire", "page": "", "keywords": ["viral vector manufacturing", "cGMP", "AAV", "Adeno-associated Viral Vectors", "gene therapy"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights Lonza's strong capabilities and experience in viral vector manufacturing, specifically AAV, for gene therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEJZK5xeIioDXBTixJzfxJ4T546dMF9QZYJ3PKXzC_B4Y60-06k2OBUA8eUVu0IDmwNTg6UsqVHEokKwZIsh__9kViGej4opzN5QZWxiPZR3OuzfUIW_w7SRj4BL3ubvXQocgFni9pMR-QecEDnnYx8hdaz1Fo0YvqmCn1jnhfNOnFWCLk6885LyXWZfDwFMG3_gRuQkEg=", "source": "Lonza Expands Cell and Gene Therapy Portfolio - Contract Pharma", "page": "", "keywords": ["AAV production", "HEK293 cells", "gene therapy vector production"], "bucket": "aav_lv", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lonza launched TheraPEAK 293-GT Medium optimized for AAV production, indicating active involvement in AAV manufacturing support."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHdQ8Pzdtg1FGzbolCJiOL5RSuFSwTCPtswTCuZCpKsdJj7M3bDEqIEZBIdu_bw7EWNJd7243sYk_a1Ofmw-p-pVAWr_eM9pduDUwmWET7JdxFf66JVCGkCMo6Ziza4iteiLqzYTmvD7RLb_vP8tEGiFI-N3uCuG1CgjjNF92unHoWIjqcVBsdnPEHSs86788=", "source": "Viral Vector Manufacturing Market Size and Forecast 2026-2031 - Mordor Intelligence", "page": "", "keywords": ["AAV vectors", "viral vector manufacturing market revenue", "2025"], "bucket": "aav_lv", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "AAV vectors delivered 72.18% of the viral vector manufacturing market revenue in 2025, providing a benchmark for AAV's share within gene therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHdQ8Pzdtg1FGzbolCJiOL5RSuFSwTCPtswTCuZCpKsdJj7M3bDEqIEZBIdu_bw7EWNJd7243sYk_a1Ofmw-p-pVAWr_eM9pduDUwmWET7JdxFf66JVCGkCMo6Ziza4iteiLqzYTmvD7RLb_vP8tEGiFI-N3uCuG1CgjjNF92unHoWIjqcVBsdnPEHSs86788=", "source": "Viral Vector Manufacturing Market Size and Forecast 2026-2031 - Mordor Intelligence", "page": "", "keywords": ["Asia-Pacific", "viral vector manufacturing market", "CAGR"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "The Asia-Pacific viral vector manufacturing market is projected to grow significantly, providing context for Lonza's APAC operations."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHSqtImJe5ZRPxGLaQuMmce20jjiFo3q3kiYegAwS4FZBTZvYpubCwJLBaG0liRCiZOR_vAmOi2rLlW1jL7RjWeHYUhpd_1fhk8MGNFIoz0KnV_ptF4GE8OGInXujn_SFx_DEao1TE=", "source": "\u200b\u200bLonza Investor Update 2024\u200b Outlines Strategy, New Organizational Structure and Guidance", "page": "", "keywords": ["Specialized Modalities", "Cell &amp; Gene Technologies", "mRNA", "Microbial", "Bioscience"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Mentions 'Specialized Modalities' business unit, which includes Cell &amp; Gene Technologies, operational from Q2 2025."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGBrhsZwLr1Qr5i6_kr-juWwHV8n6IwUrr2ph5VrltTLrx3yZihpL1-BRDaC0a8Vv1eGiKvQqtNKKfGLpRVBZ3fFACLizwJhTCJJ-huKIClitZMVVNEGt6smH-JPD8Zkz0i3NUXggk=", "source": "Lonza Delivers Strong Profitable Growth in Full-Year 2025 and Successfully...", "page": "", "keywords": ["Cell &amp; Gene (CG)", "softer performance"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Notes a 'softer performance' in Cell &amp; Gene (CG) in FY 2025, indicating potential fluctuations in revenue contribution."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFyhOj3Eld4cK0YBkiMMzVyz4vhKzaleQhVeDcSoOm_e7M5fcjQB7qiaypE8JYrQGldFV512a9Mi8Zgcvi633NNhZ3uVOZgJjOypyzH32H1a_S11L3Sf4UCFym4iJDNDt5CaCdYJcGwO7ZvBJEiuZUTspCfS1_v1jgP1jrfGB67ljfrYzFyElO5lKpDiLtulF8YE--NTIwScLtDdb4ShUUHizxrsTbEuU2HQkqucJIK1ho5Sdf5myk=", "source": "CDMO pulse check: Lonza posts major sales rebound as Samsung Bio keeps revenue growth rolling | Fierce Pharma", "page": "", "keywords": ["cell and gene technologies", "underperform"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Mentions that Lonza's cell and gene technologies continued to underperform in H1 2025, suggesting a lower revenue contribution compared to other segments."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEpGk9he_U9cbeq8jXw5yg8V2DOrvDK9JnfKZNdpKNod4N1rz37ooYyA2trqKehsIbZGmEXB4uvm4cJ-BmwssK46reYV9WihgsiPGh87cdVuHyZBoi8qNXZdINbcIKGqXMdn0gZPA64e-ISU8KZZuEyI9BneGHx6sC5sVam-jUd4sJgwMvjiWNU7g==", "source": "Annual Report", "page": "", "keywords": ["Cell &amp; Gene", "softer performance"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Reports a 'softer performance' in Cell &amp; Gene in 2023."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFuM5jzfd3nAL_JGH842o0221psRHYa9rUgLCDjQ7Wqoi7-krKGqzwLukN1RmGGh1BUQ8YS_4AXb3wSE2iXuZtP3Uw0fU1DUdEEMWh0n-3BrpOI8X0orJIKaJhi2a9dhXit7olItN0sUfkvJrd6", "source": "Financial Highlights - Lonza", "page": "", "keywords": ["sales", "CDMO services", "cell and gene technologies"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lonza reported CHF 6.6 billion in sales for 2024, with strong demand for CDMO services including cell and gene technologies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHSIUJrepqYnuMtfK0N2v_4l2XA1640KMlKZW0Inaf77TbE5h7eOFOtgoRsne2P1XSll7bDSuqot0iGtqWfcWC6aq4LVYa6p67Lfw86YIBxY8fG7ttm5DyZmUxcYTnhIvzYlxOynMCLihlnVhYFPvvVBa24UJrBj3CGp8l3bEGiNt-Uq4Lz-qsfbCI8SfWaSLK79Nd1DwbN9Rn6OPe5UBlbowl_NVkrccUNDSY=", "source": "Development of high-performing stable producer cell lines for therapeutic AAV vector manufacturing - Lonza", "page": "", "keywords": ["AAV vector manufacturing", "stable producer cell lines", "HEK293 cell based"], "bucket": "aav_lv", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Details Lonza's development of high-performing stable producer cell lines for AAV vector manufacturing, indicating advanced capabilities."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE4MBhC78WohbHYTbQJsbTA-bJD8-DYRJ74wvJirDZclPsjYktjlrNONcrkISEYdpbAshH7BJuyDQYdG5nJjeahPkyAVthdpHxLBubnh2puzEjOgvXjuhWMDb7VkPDaPWI-sF0mJryf3mNCnHelLQEtIrREqq2j5N4dtQsc8t4zje4FapJyizuAapFg8AHcYE24k3M82tq8KWfeIQ5QObfDgY3oMTI=", "source": "Cell therapy weekly: initiative to expand APAC cell and gene therapy development", "page": "", "keywords": ["gene therapy", "manufacturing agreement", "Genetix Biotherapeutics"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lonza extended its commercial manufacturing agreement with Genetix Biotherapeutics for a beta-thalassemia gene therapy, demonstrating ongoing commercial gene therapy manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGLemyx0i4cFwZgd74ZxordT8pUDmqoBubkdc4wZ0C-aMthUj4N2slSf8E0vHILyaG8ToCXEX-K8iTnu9UMYGKUR43SaGPhK0rx92Fcwr_iW2F4dMFqPbcmC2z_IB6PoH3Yrvk=", "source": "Lonza 2024 - Annual Report", "page": "", "keywords": ["employees", "global development and manufacturing sites"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Lonza has &gt;30 global development and manufacturing sites, supporting a broad CDMO presence."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGd3uNYhLyOsycsPJugHdtN_DcxBWdQdEr-Gyhwsmtb13F7TKGY1tLt5Q0ULLkAQpzoNxzI0B-xLKis1s5Be4CmS7MM0my6naWzZat9yMMLqxZQ1hwT-gqYFZbXCPEBHvGVLd1wHiw=", "source": "Lonza - AnnualReports.com", "page": "", "keywords": ["global sales", "CHF 5.9 billion", "2019"], "bucket": "gene_therapy", "confidence": 1, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Provides historical global sales figures for Lonza, used as a basis for overall company size."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHdQ8Pzdtg1FGzbolCJiOL5RSuFSwTCPtswTCuZCpKsdJj7M3bDEqIEZBIdu_bw7EWNJd7243sYk_a1Ofmw-p-pVAWr_eM9pduDUwmWET7JdxFf66JVCGkCMo6Ziza4iteiLqzYTmvD7RLb_vP8tEGiFI-N3uCuG1CgjjNF92unHoWIjqcVBsdnPEHSs86788=", "source": "Viral Vector Manufacturing Market Size and Forecast 2026-2031 - Mordor Intelligence", "page": "", "keywords": ["viral vector manufacturing market", "USD 2.95 billion", "2025"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Provides the overall market size for viral vector manufacturing, which is a key component of gene therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEpGk9he_U9cbeq8jXw5yg8V2DOrvDK9JnfKZNdpKNod4N1rz37ooYyA2trqKehsIbZGmEXB4uvm4cJ-BmwssK46reYV9WihgsiPGh87cdVuHyZBoi8qNXZdINbcIKGqXMdn0gZPA64e-ISU8KZZuEyI9BneGHx6sC5sVam-jUd4sJgwMvjiWNU7g==", "source": "Annual Report", "page": "", "keywords": ["viral vector manufacturing", "capacity", "scale-up", "purification", "quality control"], "bucket": "gene_therapy", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights the importance of manufacturing capacity and output for viral vectors, an area where Lonza has expertise."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGLJwxtvofJyc9tc0GE7yXtxoVAVAl1_5o-GU3qK-TP8x4QNK1kk1jLVnyNVYMGw_QYJAnWpiEQUHukKwTzuGEPuMi6_h-Kn9ZFeaSsoEovxJuc5mk1taga5szTiPdUc1YhIaITmzztO2RJyV1qG7nqGJLctue6ZEEnUG5QGIkW7uG6NvZJ-4YjAj8H0LJ655WrBPg0", "source": "Corporate Overview", "page": "", "keywords": ["Pharma&amp;Biotech segment", "cell culture therapies"], "bucket": "stem_cell", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Mentions Lonza's Pharma&amp;Biotech segment as a leader in advanced cell culture therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFJpTuuQoJC0Z4IpreBhf7g_-SQlsN8rpP7OwYlpvOhYYEjBbgvgzjzv0g7xvV9Ycvye-PFZ-gMwe26eCgYp9QlZAJuPjVTI61Sk9iBjcWTJIe75Q3TMUaz__CAL8tdwWP3-FwVa3Ry1DTGAtq2XXW1RJkN-tI4Ov9iaZsie4dD7cBYiDBsN9HJ6t2PTCx0_w==", "source": "Lonza Annual Report 2024", "page": "", "keywords": ["iPSCs", "MSCs", "NKs", "allogeneic cell therapies", "autologous CAR-T", "TIL", "HSC", "TCR", "T-reg gene therapies", "viral vectors", "AAVs", "LVVs"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Explicitly lists a wide range of cell and gene therapy modalities, including MSCs and iPSCs, demonstrating comprehensive capabilities."}]</t>
         </is>
       </c>
       <c r="F4" t="b">
@@ -702,46 +714,184 @@
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>81.18000000000001</v>
+        <v>141</v>
       </c>
       <c r="I4" t="n">
-        <v>40.59</v>
+        <v>40</v>
       </c>
       <c r="J4" t="n">
-        <v>60.89</v>
+        <v>90.5</v>
       </c>
       <c r="K4" t="n">
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>81.18000000000001</v>
+        <v>195</v>
       </c>
       <c r="M4" t="n">
-        <v>40.59</v>
+        <v>55</v>
       </c>
       <c r="N4" t="n">
-        <v>60.89</v>
+        <v>125</v>
       </c>
       <c r="O4" t="n">
         <v>1</v>
       </c>
       <c r="P4" t="n">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="Q4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R4" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="S4" t="n">
+        <v>269</v>
+      </c>
+      <c r="T4" t="n">
+        <v>70</v>
+      </c>
+      <c r="U4" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "webSearchQueries": ["GenScript ProBio annual report", "GenScript ProBio investor presentation", "GenScript ProBio earnings release", "GenScript ProBio regulatory filings", "GenScript ProBio official website", "GenScript ProBio CDMO advanced therapy", "GenScript ProBio viral vector manufacturing", "GenScript ProBio gene therapy manufacturing", "GenScript ProBio stem cell manufacturing", "GenScript ProBio AAV manufacturing", "GenScript ProBio lentiviral vector manufacturing", "GenScript ProBio GMP manufacturing facilities", "GenScript ProBio revenue advanced therapy", "GenScript ProBio biologics CDMO revenue"]}</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GenScript ProBio</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>["GenScript ProBio's total revenue for advanced therapy manufacturing is estimated as a significant portion of its reported 'Biologics Development Services' (ProBio) segment revenue, which was $388.7 million in FY2025. This is based on the numerous mentions of CGT projects, viral vector manufacturing, and cell therapy services within ProBio's offerings.", "It is assumed that 60-80% of ProBio's FY2025 revenue ($388.7 million) is attributable to advanced therapies (Cell and Gene Therapy), given the balance of CGT projects (60) versus antibody &amp; protein drug projects (41) in 2025. This yields a range of $233.22 million to $310.96 million for total advanced therapy revenue, rounded to $230-$310 million.", "Gene Therapy Manufacturing revenue is estimated to constitute 80-90% of the total advanced therapy revenue. This is due to the strong and explicit focus on viral vector (AAV, LVV) and plasmid DNA manufacturing, which are core components of gene therapy. This yields a range of $184 million to $279 million, rounded to $180-$280 million.", "AAV/LV Viral Vector Manufacturing revenue is estimated to be 70-85% of the Gene Therapy Manufacturing revenue. This is supported by the dedicated new facilities for AAV and LVV, the specific platforms, and the frequent mentions of these modalities. This yields a range of $126 million to $238 million, rounded to $125-$240 million.", "Stem Cell Therapeutic Manufacturing revenue is estimated as a separate bucket, representing 10-20% of the total advanced therapy revenue. While 'cell therapy' is often mentioned alongside 'gene therapy', direct evidence for manufacturing of *therapeutic stem cells* (beyond viral vectors used in cell therapies) is less granular. The partnership with Comprehensive Cell Solutions, which includes cell collections, apheresis, and cryopreservation, provides the most direct support for this category. This yields a range of $23 million to $62 million, rounded to $20-$65 million.", "The 'total_advanced_therapy_revenue' range is calculated as the sum of the 'gene_therapy_revenue_estimate' and 'stem_cell_revenue_estimate' ranges to ensure consistency: ($180 + $20) to ($280 + $65), resulting in $200-$345 million.", "All revenue figures are in USD millions."]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GenScript ProBio</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>[{"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGoFXu9m0tsuK3P0xWX2A8VRYvD-adqlo3RlkipTDdhWCgWe1NrR9Q8Lyu7aL-oORuUefNzrHmAH0BCQidv4cYMnc4oBpJ1oFo9egJglyKOfH11ChMhvsSTUn-eqXfzxWXIk30zGFfj9T2JrrvSXQBK5XzEIC32dtBuPX_dOh1ml15xTNlsazD9EcGKygSeY_FQpbb5QRxQwPeMblXkT1Cq57ijaww7UpU", "source": "Fierce Pharma", "page": "", "keywords": ["GenScript ProBio", "gene therapy production plant", "NJ", "plasmid DNA", "viral vector-based therapies", "CDMO", "manufacturing facility", "Hopewell, New Jersey", "cell and gene therapy production"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Reports the opening of a new gene therapy production plant in NJ for plasmid DNA and viral vector-based therapies, highlighting GenScript ProBio's manufacturing capabilities in cell and gene therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE1ns9eH0OXvNdD-NfkzVKN2sLYSqqa__4vGQ0RFE1LafLd2DXAh0T3RoS0qKrmA1KTa9EUo25mM1kRwpoo1mpqNqCZtWpp2UzbqO2G0XwZhjB0pqcHNA==", "source": "ProBio CDMO - Biologics and CGT CDMO Services", "page": "", "keywords": ["ProBio", "GenScript subsidiary", "end-to-end CDMO services", "biologics", "CGT", "plasmid", "viral vector", "mRNA", "GMP", "IND support", "cell &amp; gene therapy manufacturing services", "AAV", "lentiviral vector"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "GenScript ProBio offers end-to-end CDMO services for cell &amp; gene therapy (CGT), including plasmid, viral vector (AAV, LVV), and mRNA, with GMP and IND support."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFwkaVPZfmqKQZYKVkLH2tqCWy4oQgpNUAXM8s_6yiUMXAAxyEMdPMbO_YOwygEMtT7mOerjGbgEYTKRLH7hFHkuZ4nhaEKkhAFlBluP-Lg6grp_K8H4apDJm9nIN85kXSf4lKF1qWII9kx0iXAVHIVmcOf8NxRsSLMxjYx_l9CxQg4BCFHX5MDuO-Hq6nRXLe78vleSWXc55_JbjU1yTKQ1Rxv-lrpPTuMKQ8rKdkBxyvhN-0rPmAiWR5hMVhsVZkB7uGu9CnPF-kegbqnIsHcprOYvmf_daSDGE0FpBRRoWIuHr_MkAJE8ujmML9gWbVzDOPz5TkOcVTzeiHP61xWI3fQ_qVPCaccN6H1a5eZQ3yF25h6ySKe", "source": "GenScript Biotech Demonstrates Profitable Scale and Strategic Leadership in H1 2025, Establishing Clear Industry Leadership Through Accelerated Growth and Innovation", "page": "", "keywords": ["GenScript", "biologics development CDMO services", "ProBio", "revenue", "US$246.9 M", "H1 2025", "511.1% increase year-over-year"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 246.9, "range_low": null, "range_high": null}, "notes": "ProBio's revenue for H1 2025 was US$246.9 million. This is the segment revenue that includes advanced therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHtvaJ4ASNbH9obqfxFheG6dKJ5JQzkubZxiGHc7gDADsQlF_XzZb2E-Ai70v4ZTYpmQFBn0gbi6cYbO02GLg6dU2mR7th0ishtbFsaa9tDiuMJw8txO2b7rcSKB-a2MrWplnQJwqqHX4BFkhcUBn9CmZuZhGwJsV9pnrao6gdKOTlzn7kjMP39Ss7_aWhfk134R1jgXlCXtVw65tU1OWRzuVmWvPZt9hdEs_WfHBm5XU2Ow5MYlugQSvE8H02lr0ynA1kHS8pthUw==", "source": "GenScript ProBio Opens China's Largest Commercial GMP Plasmid Manufacturing Facility", "page": "", "keywords": ["GenScript ProBio", "GMP plasmid manufacturing facility", "Zhenjiang, Jiangsu Province", "one-stop service for plasmids", "cell and gene therapy mRNA drugs", "viral vectors", "separate production facilities for plasmids and viral vectors"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights GenScript ProBio's GMP plasmid manufacturing capabilities, which are crucial for cell and gene therapy and viral vector production."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHzDSi3vtLSiIvZFBCTOe1SQdxMIGvq0vPr5LUuXUyrEW5Wv5oHmOdLXXmKwmffE5qVc8Nz7RI5YtSW7lMCil4jNXsVLAprj0FfTDSeXDYfPoDlEBvM8-gyp4jlECxeAZKm9rV-vyu78dfPfkXdP1nRJgMNAZNOcMpJYLaf-hgqgQrHz067I2HeDUFSFGPjmszLWg2LQNTYx-R-386HwdVT_mqjB6D1YpDQgUP7wUJMJKBjsceDtEMVbsfmDS6uCuTVwKw0_JRZ6rlkg8rkUun9Zj04uoftuYHirw==", "source": "GenScript ProBio Signs Viral Vector Manufacturing MOU With Curocell for Next-Generation CAR-T Therapy - Business Wire", "page": "", "keywords": ["GenScript ProBio", "viral vectors", "cell and gene therapy (CGT)", "GMP production platforms", "CAR-T therapy"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "GenScript ProBio specializes in viral vector manufacturing for cell and gene therapy, including CAR-T therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGakm5EGXaJtfW9oSw1GgZyITjRB22AGZ9SMHFZZzB4ha-3DSAxa0Js_ssi9v6dQiuL2IOY14YuxMkXZIzFnZmnA0A6PZXBx3zd8NPpA9mhCkSC4MJxPxg15X7DaYLf7Nxay9Bm", "source": "GenScript Biotech Reports First Half 2021 Results - FirstWord Pharma", "page": "", "keywords": ["GenScript ProBio", "biologics CDMO business", "USD 31.5 million", "revenue", "H1 2021", "65.8% YoY increase", "GCT CDMO business"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 31.5, "range_low": null, "range_high": null}, "notes": "ProBio's revenue for H1 2021 was US$31.5 million, with growth driven by GCT CDMO business."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHuuvNS79gf_kE3Uv4s89VcpyInWbbJas-uuCx7eVLKnUJxVNshS7w10D4p8QG8fXtIsiHKuvVObdoOqao9cFgoWwy1mHJqiAo_PFwEV23N32p9lFXGCL3FRfNMhgdROBXzCYFW3thpYJyC2CZYimOnlZhs4ECnVSUCvfGxVYhJLt0-RH9NmiNLwYbdPVyAehqAWtvhrvAA1igbhGkG7fIU", "source": "GENE AND CELL THERAPY", "page": "", "keywords": ["lentivirus manufacturing", "GMP facility", "gene and cell therapy", "lentiviral vectors", "adherent culture system", "preclinical and clinical supply", "lentivirus services", "1200 m2 GMP facility for virus manufacturing"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Details GenScript ProBio's lentivirus manufacturing capabilities, including GMP facilities and services for gene and cell therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE0Zitlof5rLnaVnnqug49DHucHYjE6NuVEbKQ7F1qlp8Bi7gdAR6a4aEbzC3UgmQd2WmsulTxNzLSAlsQudp_unCEJGkAdx7XkxP-TByPXrru5ArP3_hhFz36yo3D4D1TYpnJ_7bloWLNzsLz-hf_kmD_b8sGiicDrimjB_-LyMojK6YBD4b0xcDSqf-OKxc9OkdflcBd4zCwzNb15rkuX1uTqrTtG_VRDEtsL_P5vcMcg6TRxCcfzmqDVEA==", "source": "Scalable Lentiviral Vector Manufacturing Using Proprietary Suspension Cell Line", "page": "", "keywords": ["lentiviral vector manufacturing", "suspension cell line", "gene and cell therapy", "viral vectors"], "bucket": "aav_lv", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights GenScript ProBio's expertise in scalable lentiviral vector manufacturing using suspension cell lines for gene and cell therapy."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHH_aUonsXWDWvOLmtmR0hSLH94JvaABMH-TT5i-kmaLvCho5pf1S7mZa1OTIUEX5YPc3sS-ihgoJJ-vVhpkBL2GkYjTOGLH_OZh-WsbBZGApip3XQyIZzX1hGH9nqYLecLAXQubtHfKEhS8Wy_SUWdfgZa5BCtnuUnjIT7g8Rvt8p0_roy3SfNPGfO2fhH16TemhJ7bQbIwmAMFwSjDA==", "source": "ProBio Opens Flagship U.S. Plasmid &amp; Viral Vector Manufacturing Facility in Hopewell, New Jersey to Advance Cell and Gene Therapy - GenScript", "page": "", "keywords": ["ProBio", "Hopewell, New Jersey", "GMP facility", "plasmid DNA", "viral vectors", "AAV", "lentiviral platforms", "cell and gene therapy", "GMP AAV manufacturing", "GMP LVV services"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Announces the opening of a flagship U.S. facility for plasmid and viral vector manufacturing, including AAV and lentiviral platforms, with GMP AAV manufacturing expected by Q3 2025 and GMP LVV services by Q1 2026."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGkDeWPX5hR9vwB5t5EDG3MDpoFnppto9LNME5joxCf6VK31xOkH_8pud3-0spn4ve6t3jdWqOwXYtJ0nR4z-m6z86KSpkkVp9QQRwUl4YVWqCjYe9nbCngFw83aN_ZcohOzc4R9t-ytOnipUSfkww-RDV_iPfOKq1_eRZxZEEUabnsSuJqsuKx3CHaqfgtfR1izhfEh0pyb21YJQ29mxwqgETozO7iAzalFKL0Og==", "source": "GenScript Biotech Demonstrates Profitable Scale and Strategic Leadership in H1 2025", "page": "", "keywords": ["GenScript", "biologics development CDMO services", "ProBio", "US$246.9 M", "revenue", "H1 2025"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 246.9, "range_low": null, "range_high": null}, "notes": "Reiterates ProBio's H1 2025 revenue of US$246.9 million for biologics development CDMO services."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGDaR1GSMGaIAg1_TVnKyXdoJhVP_qhZnpDP6rEAoJbK7MydVlDy98I6_avb8a74E_JG-hdnCoPyTCgcJm0biK_APQRtaEooQn7iu7oJfTSRZ7L-EAAGmMSig5pHGgg2aPk9Y_bE5p3Dqg7mB_AZ0fkSbNWzKdr9KxXDS2GIJGhxq53-1tEZvpApMmfj04=", "source": "GenScript Annual Report 2023", "page": "", "keywords": ["GenScript ProBio", "CDMO division", "integrated services", "antibody/protein-based therapeutics", "cell therapies", "gene therapies"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Confirms GenScript ProBio as the CDMO division providing services for antibody/protein-based therapeutics, cell therapies, and gene therapies."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHNui5z0WSrmqm615xax51I9Xk8ZJyY7Mwe_dc4J6AJ187kmmAtrxA7hN0FxMECz0zTkApxTnbOx6L8ZVBcKhsqPWM8VhxSr8tulxKHcBHDPAImDyHyNhUVm3ooJa2ecrR9UIG1Bf616rRQgc89aIlUyaHTcPsSnSq-EZomoR0JZ-NURvxlMTSbP4yJNMaPGg==", "source": "GenScript ProBio USA Inc - BIO International Convention", "page": "", "keywords": ["GenScript ProBio", "biologics CDMO segment", "gene and cell therapy", "total gene and cell therapy solution", "CMC of plasmid and virus", "IND filing", "clinical manufacturing", "commercial manufacturing"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "GenScript ProBio offers a total gene and cell therapy solution covering CMC of plasmid and virus for IND filing, clinical, and commercial manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHdyMwAL59o3m286yoxHuKmmTSPTPAvfTgpOBzbPY80jC_8QSvRbfKiKDLWg4XzUBeLtYGmEAw7dObBut6uBX6aIHM4EUQ9CYtqRPGfIL2widRF_H6e-9J_BzG8XrnhAnMgvipc3QCYNBjk3OZv9H9cw36wuIH1yYHixdTjcI5oMadtRSqTfTpKW4afMCt6qFQC0g9tl_X50dCQNEw1", "source": "GenScript reports strong fiscal 2025 results from platform strategy", "page": "", "keywords": ["ProBio", "revenue", "US$388.7 million", "FY2025", "309.1% year-on-year", "60 cell and gene therapy CDMO projects", "20 new IND clearances across CGT programs", "GMP manufacturing capabilities"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 388.7, "range_low": null, "range_high": null}, "notes": "ProBio's revenue for FY2025 was US$388.7 million, with 60 cell and gene therapy CDMO projects and 20 new IND clearances in CGT."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF6nPBKxTXt1sQSkRwuS4jcJ_8DcRoVmA2uJouxxCiLELujvgoZHzRkISGwzknae8osKFc2Y2PpW84TsQ4ZBN0snvfwIzoLBC9SS9YejHdx_dO1U6GegjnVUiYxAtt94MOu9gR_iMoGyztgEk35h1AnNOln4dm4jy7JXvnWppGCTW8UN68RhZP6R-lBjAvJHzqdimERZdWwZC6kLe5kdBhRzZvRbhgF3qr_NpfzuZdMn-WOI_7JKk8LF_433y15JmfjuGVkgjnZ7_LVsHiFaGfyNkSBtpbI-P-48S9MXZ7-a5rnQkD1tHIVf7rPRGz9MdykiLMzVxOs", "source": "GenScript Biotech Corp Reports Strong FY2025 Results as Integrated Platform Strategy and Global Execution Drive High-Quality Growth - PR Newswire", "page": "", "keywords": ["ProBio", "revenue", "US$388.7 million", "FY2025", "60 cell and gene therapy CDMO projects", "20 new IND clearances across CGT programs", "GMP manufacturing capabilities"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 388.7, "range_low": null, "range_high": null}, "notes": "Confirms ProBio's FY2025 revenue of US$388.7 million and its significant involvement in cell and gene therapy CDMO projects."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFLAIuE7uI4ZtRmuJJLjDIpr1vRorG-Cm4o5hTb_F1lRWE502vja2AYoJmVIFOvJFPYT5RbTCsVmp1HHblRKOUkq2FtFhxEn6PzwR9kMTuO0p_-ixxI-znvy5lMcVcEj9DpDMYXp21vpAgOVbsgdXVIrT5jd6xzf3eb27o7UUtuDafQhz010GLGsG3G8oYmPg==", "source": "AffyXell expands its strategic partnership with GenScript ProBio - Avacta Therapeutics", "page": "", "keywords": ["AffyXell", "GenScript ProBio", "cell therapies", "mesenchymal stem cells", "viral vectors", "process development", "production"], "bucket": "stem_cell", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "GenScript ProBio's partnership with AffyXell involves cell therapies based on mesenchymal stem cells and includes the production of viral vectors for these cell therapy products. This indicates involvement in stem cell-related manufacturing, though often linked to viral vectors."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF7NF0x4EgzpCrqEykzu9jqtzBVS9oNLaXR5fPE3UZIHhEYjf0QgVLK-x5tL6DMCPnURh5MuiIdctrXPDYdDA0HaUxtJrYd_wDSRHAddFEBUn_cofKnP0KpL9sEaACBmc7m7mEOSVoMpM4CsnPLhXKXp8OyMhyTkjG-ClYj4mBs0OhbWdaaO9esbRxYk2RnAT-QvpmEAcCgRq4_saX79w3iPDi3_gy4hHG_XQNh8WhXNOpdqSvEQIJF8lBQKHdm8hneij-crWvPNI2mSRGv4XiTQgNxCZiILw6QNvejFXfxD16Gur_N3j_wS2ySirlWLpGSwm1ToXb8POvmMjRv0eEnWrC-H8W1ov0y_muSyYkIJPDZWTCOx5c_hGMbuByGJJ8AqJukC3eb8uz05dqBCu5oGmHWTh2wlK1Mine6RQ==", "source": "GenScript ProBio and Comprehensive Cell Solutions, a Business Unit of the New York Blood Center Enterprises, Form a Pioneering Partnership to Expedite Cell and Gene Therapy Development and Manufacturing", "page": "", "keywords": ["GenScript ProBio", "Comprehensive Cell Solutions", "cell and gene therapies", "cell therapy services", "cell collections", "apheresis", "cryopreservation", "CAR-T therapies", "viral vectors"], "bucket": "stem_cell", "confidence": 2, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Partnership to expedite cell and gene therapy development and manufacturing, offering a comprehensive suite of cell therapy services including cell collections, apheresis, and cryopreservation of final therapeutics. This directly supports stem cell therapeutic manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH_blLXdVAbKjuigPRc4tTeltQ9nT_3i_F3GT4oHhY8ahc1MA5wTKKhOb3wFi0mDa_40dkecC7o7DBS9m51LkfuJEdWW7BW0CLMryQMvNLw7dX-7HcRpH5cjOujGerkFE5nsHULVYgkLH-Ce_zoV-5lUpIdqcpG9hgY2rFpDkWsrEiwUZlZdxflYtKudWETpqEc8z8=", "source": "2025 Annual Results - GenScript", "page": "", "keywords": ["ProBio", "60 CDMO projects in 2025", "CGT New Projects", "Viral Vector", "Plasmid", "mRNA", "Integrated LVV CMC platform", "Upgraded AAV platform", "1st commercial plasmid &amp; LVV mfg. project"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Highlights 60 CDMO projects in 2025 for CGT, including viral vector and plasmid. Mentions integrated LVV CMC platform, upgraded AAV platform, and the first commercial plasmid &amp; LVV manufacturing project."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE5SMoHgEfyPQzjd3mlu4wdURJcmb104SQ0gDNvlts2Vq_vDjPnOHt0x8FLUxvqgwzz3LhAWstgwXFywwYLJ10WN-uUiU-kWlj8lhwWedEvaY1yRpd-XfP94lBuWXT8ylO1RsvzDK9QZc59H2-ePNowguF_1Z9c9p3G2fdATwIr0i93qtavfY3hmqVo-SrFIlrBTWdqHtINfEWMfxLkXq22SDIPPxCSrFr7kA==", "source": "Contract Manufacturing of Plasmid DNA Under GMP-Compliance", "page": "", "keywords": ["Plasmid DNA", "GMP-Compliance", "viral vectors", "LV", "AAV", "gene and cell therapy", "raw material", "drug substance", "drug product", "CAR-T projects", "pre-clinical manufacturing", "early stage clinical", "GMP manufacturing"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": null, "range_low": null, "range_high": null}, "notes": "Details GenScript ProBio's GMP plasmid DNA manufacturing services, which are used as raw material for viral vectors (LV, AAV) in gene and cell therapy, and for CAR-T projects."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEqYYWA7Huc-jr3QSsDoOpUuUxA9RDSy1ig54TqtUEkFoa9zaiJdPSssNK2ke-pRRBACqaSNaneHP2qzr6VvfoSN9o-rYam9hebeC2ZqoGxAxoDKqTfksaQmbpBYrxkJANCXffIpdX-o2ZcdJxbe4KjdN_d_hwB6Yt_Hd-zFn3jduKE30pJl3a8Gm0Xw5gi_Vl4VnZsCpOA1Wc", "source": "2025 Annual_Results_Management_Remarks - GenScript", "page": "", "keywords": ["ProBio", "2025", "total revenue", "$388.7 million", "FFS revenue", "21% organic growth", "protein &amp; antibody", "new order intake", "cell and gene therapy"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 388.7, "range_low": null, "range_high": null}, "notes": "Confirms ProBio's total revenue for 2025 as $388.7 million and mentions cell and gene therapy as a key area of growth."}]</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>240</v>
+      </c>
+      <c r="I5" t="n">
+        <v>125</v>
+      </c>
+      <c r="J5" t="n">
+        <v>182.5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="n">
+        <v>280</v>
+      </c>
+      <c r="M5" t="n">
+        <v>180</v>
+      </c>
+      <c r="N5" t="n">
+        <v>230</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q5" t="n">
         <v>20</v>
       </c>
-      <c r="R4" t="n">
-        <v>35</v>
-      </c>
-      <c r="S4" t="n">
-        <v>131.18</v>
-      </c>
-      <c r="T4" t="n">
-        <v>60.59</v>
-      </c>
-      <c r="U4" t="n">
-        <v>95.89</v>
+      <c r="R5" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="S5" t="n">
+        <v>345</v>
+      </c>
+      <c r="T5" t="n">
+        <v>200</v>
+      </c>
+      <c r="U5" t="n">
+        <v>272.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>{"searchEntryPoint": {"renderedContent_omitted": true}, "groundingChunks": [{"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEynqkJkFFqt7UzStIZrP-Pl0_J5PMF0vaMpPUVjOHcqr8kkNBTVAbB1aoSNE05f19Zk3ZrrIw-Y0kZz7LPEFszv4BkHGj_f7mdBOm3YvuWVfuQGhhqrnaFgrIh9XViGtYnsFLBV5Glhzh9mcy7l2tfzs84Su-8sm4=", "title": "wise.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFmsP8mEcGc6K1fRIXdb1OfGYQw6etttoS6Fxx_P6tWb1sQcKg79ea0KdWt0Pt1xjFR-uJjgbec2v9BF__5zTNjSDNrA6QEs7uJevFJYfViPVdGLha0yzWLlsKpZ8ZR8AoGhRXt2h4AlDw=", "title": "alanchand.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGj44eeP714z4jLOcFdo601-I56EZmX4nj7bk7rAZ24Gaas5LGgMVKHCguuPoaXdyAPhVE84F8OneAJM0obkrwKjE8Vc2HGBkr-ko5OGyqDFrUyDluV6jbOyqEvymjh-hng0bkN0YQD10epU0vp3_WUkjNKQQVMkeAb59ud6jjoTtmt-0homQ==", "title": "xe.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE05CPH25-M5-OGaw0pGsjOEullGtBrPF6fZD9qiv6fXTh90VD5ifRb6L_VYibPOFE3-iaTCx5v5jaV5p3seJUuRWf_xvi0KKD38iCkDicIYcxNXfYJTMWr-T4E4nm3hsoKbrBq8bbDTyj7x_6jZTX6gyeuRI7Zr0htSaFn6pmxKHFn3jKzR0dSEy1FgNI=", "title": "mtfxgroup.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHJQWtxioLeD-Vh0PllTKVZz17p4uQUS_9t6sKtTewNuxNlO81X9Ht943kdTlYGnMQZI-rKIbDX5ZUZoayPe4kJKV4baRr7Jil1CD5HEiNOxM83NpACzuK3wesnDc6k4xnOXVSECLfl_P-vc751iBrPCnQ2q3zuyjfOy_mFtAXZXrT99cnAiQ==", "title": "mtfxgroup.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGmN0WG_KAmb8NkSszmjkAmDD0IMSBad6dQ2C796tJ12jLFsYn-tmMV_FxlxWK548bNZcQiMVaPkzFBYLGTgSvFZToty2GZKed4Rl83KqAc53Dfc16rzR1AZcq7Lfs6Uoj-KWgkWJKwW16NzKG2lSrVpL4zCLQ=", "title": "xtransfer.com"}}, {"web": {"uri": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGVl70qm2UEbEI_Yedrste3-yqkeZrHRuD-5V1TJfTx68qRk7oUynsFp3jH732M-RXCZae6wKoIJWt0CEY4JjHRJL2ceRlK12i8kLwm1b1DHYQsOd7yJCH-vhu50eJhwmF_IL0NhixS347ZVhpUflOidvh3qmpGATffS2WIxvu9-x0JD6GknLzp", "title": "exchangerates.org.uk"}}], "groundingSupports": [{"segment": {"startIndex": 7396, "endIndex": 10210, "text": "- FirstWord Pharma\",\n   \"page\": \"\",\n   \"keywords\": [\n    \"Cell and Gene Therapy (CGT) field\",\n    \"Contract Development and Manufacturing Organization\",\n    \"GMP production facility\"\n   ],\n   \"bucket\": \"gene_therapy\",\n   \"confidence\": 3,\n   \"reported_or_inferred\": \"inferred\",\n   \"estimated_revenue\": {\n    \"value\": 2.81,\n    \"range_low\": null,\n    \"range_high\": null\n   },\n   \"notes\": \"Confirms OBiO's core business as a CGT CDMO with GMP facilities, supporting the attribution of overall revenue to advanced therapies and the subsequent split.\"\n  },\n  {\n   \"url\": \"https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHV4r-AlIEshUY5tl6gNnGTN4SmcoxXS1gWd2PjGREWacm3njw_OMDmYf5znr73eLcKJYz2xmRNMK8jaMveFbTVVMJ5jDhRe6GwlZhn2Nyixk0u9iXa_BrB9qjGcSdKQyrCi3CkyJfhZcUEfJ1qkygA2kpdf26PoaRmmYWmkzGVFBTLkbZQ5kzNMxBSFy8pYFPVVGKmXGlFeuALyQUTciBkrK-IHnfOOneOn3EO-JIZLT0HkZc0T1w2z2TMG9q1E1jpArtvTtNSzTiQQ9qxPOR-8LUnV2U_AuUrSg8=\",\n   \"source\": \"OBiO Technology Launches New Super Factory in Shanghai with 29 GMP-Grade Production Lines for Gene and Cell Therapy - BioPharma APAC\",\n   \"page\": \"\",\n   \"keywords\": [\n    \"leading gene and cell therapy CDMO\",\n    \"GMP manufacturing base\",\n    \"OBiO Intelli-M\",\n    \"gene and cell therapies\"\n   ],\n   \"bucket\": \"gene_therapy\",\n   \"confidence\": 3,\n   \"reported_or_inferred\": \"inferred\",\n   \"estimated_revenue\": {\n    \"value\": 2.81,\n    \"range_low\": null,\n    \"range_high\": null\n   },\n   \"notes\": \"Further evidence of OBiO's focus and capabilities in gene and cell therapy manufacturing, supporting the revenue attribution and split.\"\n  },\n  {\n   \"url\": \"https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHV4r-AlIEshUY5tl6gNnGTN4SmcoxXS1gWd2PjGREWacm3njw_OMDmYf5znr73eLcKJYz2xmRNMK8jaMveFbTVVMJ5jDhRe6GwlZhn2Nyixk0u9iXa_BrB9qjGcSdKQyrCi3CkyJfhZcUEfJ1qkygA2kpdf26PoaRmmYWmkzGVFBTLkbZQ5kzNMxBSFy8pYFPVVGKmXGlFeuALyQUTciBkrK-IHnfOOneOn3EO-JIZLT0HkZc0T1w2z2TMG9q1E1jpArtvTtNSzTiQQ9qxPOR-8LUnV2U_AuUrSg8=\",\n   \"source\": \"OBiO Technology Launches New Super Factory in Shanghai with 29 GMP-Grade Production Lines for Gene and Cell Therapy - BioPharma APAC\",\n   \"page\": \"\",\n   \"keywords\": [\n    \"leading gene and cell therapy CDMO\",\n    \"GMP manufacturing base\",\n    \"OBiO Intelli-M\",\n    \"gene and cell therapies\",\n    \"18 cell production lines for autologous and allogeneic immune cell therapies and stem cell therapies\"\n   ],\n   \"bucket\": \"stem_cell\",\n   \"confidence\": 3,\n   \"reported_or_inferred\": \"inferred\",\n   \"estimated_revenue\": {\n    \"value\": 4.59,\n    \"range_low\": null,\n    \"range_high\": null\n   },\n   \"notes\": \"Confirms dedicated cell production lines for stem cell therapies, reinforcing the revenue allocation to this bucket.\"\n  }\n ],\n \"assumptions\": [\n  \"The reported Q1 2026 sales of CNY 50.54 million for Shanghai Obio Technology Corp., Ltd."}, "groundingChunkIndices": [0]}, {"segment": {"startIndex": 10211, "endIndex": 10376, "text": "are assumed to be 100% attributable to advanced therapy manufacturing, given the company's explicit and consistent self-description as a 'gene and cell therapy CDMO'"}, "groundingChunkIndices": [1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14]}, {"segment": {"startIndex": 10377, "endIndex": 10459, "text": "\",\n  \"The CNY to USD exchange rate used for conversion is 0.1464 as of May 3, 2026"}, "groundingChunkIndices": [1, 2, 15]}, {"segment": {"startIndex": 10460, "endIndex": 10731, "text": "\",\n  \"The total advanced therapy revenue is split between 'gene_therapy' and 'stem_cell' based on the reported number of production lines in their OBiO Intelli-M facility: 11 vector production lines for gene therapy and 18 cell production lines for cell/stem cell therapy"}, "groundingChunkIndices": [2, 8]}, {"segment": {"startIndex": 10915, "endIndex": 11031, "text": "Given OBiO Technology's strong emphasis and explicit mention of AAV and Lentiviral vector manufacturing capabilities"}, "groundingChunkIndices": [3, 15, 16, 4, 17, 6, 9, 12, 18]}], "webSearchQueries": ["Obio Technology annual reports", "Obio Technology investor presentations", "Obio Technology earnings releases", "Obio Technology regulatory filings", "Obio Technology company website", "Obio Technology manufacturing sites", "Obio Technology advanced therapy manufacturing", "Obio Technology CDMO", "Obio Technology gene therapy manufacturing", "Obio Technology viral vector manufacturing", "Obio Technology stem cell manufacturing", "CNY to USD exchange rate May 2026", "current CNY to USD exchange rate"]}</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Obio Technology</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>["The reported Q1 2026 sales of CNY 50.54 million for Shanghai Obio Technology Corp., Ltd. are assumed to be 100% attributable to advanced therapy manufacturing, given the company's explicit and consistent self-description as a 'gene and cell therapy CDMO'.", "The CNY to USD exchange rate used for conversion is 0.1464 as of May 3, 2026.", "The total advanced therapy revenue is split between 'gene_therapy' and 'stem_cell' based on the reported number of production lines in their OBiO Intelli-M facility: 11 vector production lines for gene therapy and 18 cell production lines for cell/stem cell therapy. This results in an approximate 38% (11/29) allocation to gene therapy and 62% (18/29) to stem cell therapy.", "Revenue for 'aav_lv' is inferred as a sub-segment of 'gene_therapy'. Given OBiO Technology's strong emphasis and explicit mention of AAV and Lentiviral vector manufacturing capabilities, it is assumed that 70-90% of the estimated gene therapy revenue is attributable to AAV/LV viral vector manufacturing."]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Obio Technology</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[{"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFbVC7BKYUtB9UTZW0ggcTa_8IZltZyylyWhlXrPBNy7t3UZo93dM5tmjtgW7YnzPMSq3VlK1iakqrKBnsEvyhopX4oFErbq_xLe0nti58D37s1FNSZmoD7faUqFpbeWjP96GduAvI6xLPacwp4yFawb06Tn0T_4Lcb1SuHSjwaEDGEghzro_F9eCU00Ivlwf48l6owIlkEqfa-2-4ddsC85_Rh5F7qAivjIaznpj8ApPFqej97ujtEw9ExmOyUrbJAj0iZbITMae70DXS6PM6q", "source": "MarketScreener", "page": "Shanghai Obio Technology Corp., Ltd. Reports Earnings Results for the First Quarter Ended March 31, 2026", "keywords": ["sales", "CNY 50.54 million", "first quarter ended March 31, 2026"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "reported", "estimated_revenue": {"value": 7.4, "range_low": null, "range_high": null}, "notes": "Reported total sales for Q1 2026 for Shanghai Obio Technology Corp., Ltd. (688238.SH), converted from CNY 50.54 million to USD 7.40 million using an exchange rate of 0.1464 USD/CNY. This is considered the total advanced therapy revenue due to the company's explicit focus."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFZGFXtVgwCyDKopp-rUOGyAGBypk3iyGkV3_6zgNZ6Gx_eqP_EDiHJU7Mljat_8zDDmmKCvzyXcvaeoUIBacpgEmMOli8VeDbRDYgm56cfaDrcPu_ZyyuHPbyT4PzL6VVL", "source": "A new super factory with 29 GMP grade production lines for gene and cell therapy was launched in Shanghai by OBiO technology", "page": "", "keywords": ["29 GMP grade production lines", "gene and cell therapy", "OBiO Intelli-M", "11 different vector production lines", "18 cell production lines", "autologous and allogeneic immune cell therapies and stem cell therapies"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 2.81, "range_low": null, "range_high": null}, "notes": "OBiO Intelli-M has 11 vector production lines and 18 cell production lines. This ratio (11/29) is used to infer the proportion of total advanced therapy revenue attributable to gene therapy manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFZGFXtVgwCyDKopp-rUOGyAGBypk3iyGkV3_6zgNZ6Gx_eqP_EDiHJU7Mljat_8zDDmmKCvzyXcvaeoUIBacpgEmMOli8VeDbRDYgm56cfaDrcPu_ZyyuHPbyT4PzL6VVL", "source": "A new super factory with 29 GMP grade production lines for gene and cell therapy was launched in Shanghai by OBiO technology", "page": "", "keywords": ["29 GMP grade production lines", "gene and cell therapy", "OBiO Intelli-M", "11 different vector production lines", "18 cell production lines", "autologous and allogeneic immune cell therapies and stem cell therapies"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 4.59, "range_low": null, "range_high": null}, "notes": "OBiO Intelli-M has 18 cell production lines for immune cell therapies and stem cell therapies. This ratio (18/29) is used to infer the proportion of total advanced therapy revenue attributable to stem cell therapeutic manufacturing."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEAFpQV80x6gJXFzDFMv5Qt8k-58c8h9eMc8WV2MUrEjDJ8ZGvPNoaSDiASG9RrjDREVvJQ_MLIlCvCpUZ7XY0zSrvHFOHG73pENhEQkkmRbqpzUB0oORpMWQ==", "source": "CDMO Solutions - OBiO Tech, Inc", "page": "", "keywords": ["CDMO services", "viral vector", "AAV", "Adenoviral vector", "Lentiviral vectors", "Retroviral vectors", "AAV Packaging"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 1.97, "range_high": 2.53}, "notes": "Explicit mention of AAV and Lentiviral vectors as part of CDMO services. Revenue range is inferred as 70-90% of the estimated gene therapy revenue."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHEeOjpROp71aLLd0eNkUKfpiswAUwxQis3anw91mk0Bynm8k3hDzKIrDWmTO8NXaPafBDN94COErDhyD4t3z5b1Up6hZNhTcD5tHqFOfYPKYACF21w0cGkoerytgdG", "source": "Viral Vectors - OBiO Tech, Inc", "page": "", "keywords": ["cGMP manufacturing services for viral vectors including adeno-associated virus and lentivirus"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 1.97, "range_high": 2.53}, "notes": "Explicit mention of cGMP manufacturing for AAV and Lentivirus. Revenue range is inferred as 70-90% of the estimated gene therapy revenue."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEN2O2f3IdHrBkVsAFfz-0GMCjGGdOULcrBC_-W8d4RtK0-pS7au4IKMlq1PFsxYL1C_O3udRalCpWejSQE16YZj3SJdYOC6ZEVSE8-GkkyMiP_POgNz4_aCJZxZzbv5IvFyF_B1y81N1P9aTt_ZVVSMUx5m_ml4pl9S-GOvhUrI2v1LHi6221VngS3_YdNX_njOvUuz0yCYgwb02ml1Oh6hCjByKkmAgCLK6zx8InAdAkUe_U0v-seXTb2qOr_CxKYcg4C6A==", "source": "FDA Acceptance of Drug Master File Marks New Milestone Achieved for OBiO TECH of GMP Plasmid Products", "page": "", "keywords": ["lentivirus production", "lentiviral vectors", "autologous cell therapy", "allogeneic cell therapy", "stem cell therapy products", "comprehensive CDMO solutions for lentiviral vector"], "bucket": "aav_lv", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": null, "range_low": 1.97, "range_high": 2.53}, "notes": "Explicit mention of lentiviral vector production and CDMO solutions. Revenue range is inferred as 70-90% of the estimated gene therapy revenue."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFrqL4oytbedbNxIxFwnJ6aA4gZmLe3doSS7T2xlFvcczNgi3SatOki6KU3pDgJKUOYlmF9Cxxbr_LBYxlmrigs41rKw2-czi-AiNrSyBsAlAXfkKbtrf2sDwebf6E_2YvBPaM=", "source": "Life&amp;Health CDMO - OBiO Tech, Inc", "page": "", "keywords": ["Cell Storage Services", "Stem Cell Cryopreservation"], "bucket": "stem_cell", "confidence": 2, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 4.59, "range_low": null, "range_high": null}, "notes": "Direct mention of stem cell services, supporting the allocation of cell therapy revenue to this bucket."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHTmOj9mKW3Zf8VYWWGKiekX7eC-4n4z2D7tZ7odctX9gws0wv_BgolkS_DrsZpWJKweAtvpZCYFSphlP-q9ZUXaouG3RqfR1Rm8h4zCHtWBakBiXO05QjYfH9IUW2hVfarhfNS", "source": "OBiO has launched its state-of-the-art GMP production facility Intelli-M to expedite innovative and advanced therapies to patients who are in need. - FirstWord Pharma", "page": "", "keywords": ["Cell and Gene Therapy (CGT) field", "Contract Development and Manufacturing Organization", "GMP production facility"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 2.81, "range_low": null, "range_high": null}, "notes": "Confirms OBiO's core business as a CGT CDMO with GMP facilities, supporting the attribution of overall revenue to advanced therapies and the subsequent split."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHV4r-AlIEshUY5tl6gNnGTN4SmcoxXS1gWd2PjGREWacm3njw_OMDmYf5znr73eLcKJYz2xmRNMK8jaMveFbTVVMJ5jDhRe6GwlZhn2Nyixk0u9iXa_BrB9qjGcSdKQyrCi3CkyJfhZcUEfJ1qkygA2kpdf26PoaRmmYWmkzGVFBTLkbZQ5kzNMxBSFy8pYFPVVGKmXGlFeuALyQUTciBkrK-IHnfOOneOn3EO-JIZLT0HkZc0T1w2z2TMG9q1E1jpArtvTtNSzTiQQ9qxPOR-8LUnV2U_AuUrSg8=", "source": "OBiO Technology Launches New Super Factory in Shanghai with 29 GMP-Grade Production Lines for Gene and Cell Therapy - BioPharma APAC", "page": "", "keywords": ["leading gene and cell therapy CDMO", "GMP manufacturing base", "OBiO Intelli-M", "gene and cell therapies"], "bucket": "gene_therapy", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 2.81, "range_low": null, "range_high": null}, "notes": "Further evidence of OBiO's focus and capabilities in gene and cell therapy manufacturing, supporting the revenue attribution and split."}, {"url": "https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHV4r-AlIEshUY5tl6gNnGTN4SmcoxXS1gWd2PjGREWacm3njw_OMDmYf5znr73eLcKJYz2xmRNMK8jaMveFbTVVMJ5jDhRe6GwlZhn2Nyixk0u9iXa_BrB9qjGcSdKQyrCi3CkyJfhZcUEfJ1qkygA2kpdf26PoaRmmYWmkzGVFBTLkbZQ5kzNMxBSFy8pYFPVVGKmXGlFeuALyQUTciBkrK-IHnfOOneOn3EO-JIZLT0HkZc0T1w2z2TMG9q1E1jpArtvTtNSzTiQQ9qxPOR-8LUnV2U_AuUrSg8=", "source": "OBiO Technology Launches New Super Factory in Shanghai with 29 GMP-Grade Production Lines for Gene and Cell Therapy - BioPharma APAC", "page": "", "keywords": ["leading gene and cell therapy CDMO", "GMP manufacturing base", "OBiO Intelli-M", "gene and cell therapies", "18 cell production lines for autologous and allogeneic immune cell therapies and stem cell therapies"], "bucket": "stem_cell", "confidence": 3, "reported_or_inferred": "inferred", "estimated_revenue": {"value": 4.59, "range_low": null, "range_high": null}, "notes": "Confirms dedicated cell production lines for stem cell therapies, reinforcing the revenue allocation to this bucket."}]</t>
+        </is>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="O6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="n">
+        <v>7.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>